<commit_message>
feat: fullfilled data and fixed grouped data
</commit_message>
<xml_diff>
--- a/inst/app/data/CAZALEGAS_B_DATA.xlsx
+++ b/inst/app/data/CAZALEGAS_B_DATA.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://urjc-my.sharepoint.com/personal/d_lopezp_2025_alumnos_urjc_es/Documents/VISUALIZACION_DATOS/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Equipo\Desktop\MASTER_MUSA\REPOS\FootballTeamTracker\inst\app\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1996" documentId="8_{4A3C1F96-2C4F-438D-8F32-D501B0DAA150}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{124FB6D6-DD5D-42E7-9841-616103177065}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEA933F1-A961-4B28-BB09-705EB6D56ED8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{46C6BD2A-3E4B-49DE-A2D3-07FEC4388880}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{46C6BD2A-3E4B-49DE-A2D3-07FEC4388880}"/>
   </bookViews>
   <sheets>
     <sheet name="Eventos" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="871" uniqueCount="83">
   <si>
     <t>Jornada</t>
   </si>
@@ -241,12 +241,6 @@
     <t>Alexandre Galimberti Zakir</t>
   </si>
   <si>
-    <t>Gol (P)</t>
-  </si>
-  <si>
-    <t>Gol (PP)</t>
-  </si>
-  <si>
     <t>Rival - Propia Puerta</t>
   </si>
   <si>
@@ -284,6 +278,15 @@
   </si>
   <si>
     <t>Hector de la Cruz Gomez</t>
+  </si>
+  <si>
+    <t>Oleksandr Ilchenko</t>
+  </si>
+  <si>
+    <t>Adrian Alexander Vazquez Trenado</t>
+  </si>
+  <si>
+    <t>Roque Alberto Celaya Rodriguez</t>
   </si>
 </sst>
 </file>
@@ -347,10 +350,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -670,7 +669,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA997B58-975D-4006-998B-0A230432491C}">
-  <dimension ref="A1:J299"/>
+  <dimension ref="A1:J418"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="22.6640625" style="3" bestFit="1" customWidth="1"/>
@@ -914,6 +913,9 @@
       <c r="I8">
         <v>1</v>
       </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9">
@@ -2660,7 +2662,7 @@
         <v>4</v>
       </c>
       <c r="D72" t="s">
-        <v>67</v>
+        <v>26</v>
       </c>
       <c r="E72">
         <v>35</v>
@@ -2686,13 +2688,13 @@
         <v>4</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C73">
         <v>4</v>
       </c>
       <c r="D73" t="s">
-        <v>68</v>
+        <v>26</v>
       </c>
       <c r="E73">
         <v>40</v>
@@ -2802,7 +2804,7 @@
         <v>4</v>
       </c>
       <c r="D77" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E77">
         <v>60</v>
@@ -2892,7 +2894,7 @@
         <v>4</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C80">
         <v>4</v>
@@ -3182,7 +3184,7 @@
         <v>5</v>
       </c>
       <c r="D90" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E90">
         <v>65</v>
@@ -3315,7 +3317,7 @@
         <v>5</v>
       </c>
       <c r="D95" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E95">
         <v>65</v>
@@ -3437,7 +3439,7 @@
         <v>5</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C99">
         <v>5</v>
@@ -3640,7 +3642,7 @@
         <v>5</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C106">
         <v>5</v>
@@ -3692,7 +3694,7 @@
         <v>6</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C108">
         <v>6</v>
@@ -3862,7 +3864,7 @@
         <v>6</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C115">
         <v>6</v>
@@ -4181,7 +4183,7 @@
         <v>6</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C126">
         <v>6</v>
@@ -4491,7 +4493,7 @@
         <v>7</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C137">
         <v>7</v>
@@ -4694,7 +4696,7 @@
         <v>7</v>
       </c>
       <c r="B144" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C144">
         <v>7</v>
@@ -4952,7 +4954,7 @@
         <v>8</v>
       </c>
       <c r="B153" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C153">
         <v>8</v>
@@ -4984,7 +4986,7 @@
         <v>8</v>
       </c>
       <c r="B154" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C154">
         <v>8</v>
@@ -5161,7 +5163,7 @@
         <v>8</v>
       </c>
       <c r="B160" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C160">
         <v>8</v>
@@ -5219,7 +5221,7 @@
         <v>8</v>
       </c>
       <c r="B162" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C162">
         <v>8</v>
@@ -5248,7 +5250,7 @@
         <v>8</v>
       </c>
       <c r="B163" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C163">
         <v>8</v>
@@ -5306,7 +5308,7 @@
         <v>9</v>
       </c>
       <c r="D165" t="s">
-        <v>67</v>
+        <v>26</v>
       </c>
       <c r="E165">
         <v>24</v>
@@ -5511,7 +5513,7 @@
         <v>9</v>
       </c>
       <c r="B173" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C173">
         <v>9</v>
@@ -5540,7 +5542,7 @@
         <v>9</v>
       </c>
       <c r="B174" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C174">
         <v>9</v>
@@ -5685,7 +5687,7 @@
         <v>9</v>
       </c>
       <c r="B179" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C179">
         <v>9</v>
@@ -5772,7 +5774,7 @@
         <v>9</v>
       </c>
       <c r="B182" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C182">
         <v>9</v>
@@ -5801,7 +5803,7 @@
         <v>9</v>
       </c>
       <c r="B183" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C183">
         <v>9</v>
@@ -6073,7 +6075,7 @@
         <v>10</v>
       </c>
       <c r="B193" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C193">
         <v>10</v>
@@ -6247,7 +6249,7 @@
         <v>10</v>
       </c>
       <c r="B199" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C199">
         <v>10</v>
@@ -6334,7 +6336,7 @@
         <v>10</v>
       </c>
       <c r="B202" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C202">
         <v>10</v>
@@ -6695,7 +6697,7 @@
         <v>11</v>
       </c>
       <c r="B216" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C216">
         <v>11</v>
@@ -6727,7 +6729,7 @@
         <v>11</v>
       </c>
       <c r="B217" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C217">
         <v>11</v>
@@ -6759,7 +6761,7 @@
         <v>11</v>
       </c>
       <c r="B218" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C218">
         <v>11</v>
@@ -6823,7 +6825,7 @@
         <v>11</v>
       </c>
       <c r="B220" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C220">
         <v>11</v>
@@ -7026,7 +7028,7 @@
         <v>11</v>
       </c>
       <c r="B227" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C227">
         <v>11</v>
@@ -7333,13 +7335,13 @@
         <v>12</v>
       </c>
       <c r="B238" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C238">
         <v>12</v>
       </c>
       <c r="D238" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E238">
         <v>66</v>
@@ -7365,7 +7367,7 @@
         <v>12</v>
       </c>
       <c r="B239" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C239">
         <v>12</v>
@@ -7397,7 +7399,7 @@
         <v>12</v>
       </c>
       <c r="B240" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C240">
         <v>12</v>
@@ -7423,7 +7425,7 @@
         <v>12</v>
       </c>
       <c r="B241" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C241">
         <v>12</v>
@@ -7631,7 +7633,7 @@
         <v>12</v>
       </c>
       <c r="B249" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C249">
         <v>12</v>
@@ -7749,7 +7751,7 @@
         <v>13</v>
       </c>
       <c r="B254" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C254">
         <v>13</v>
@@ -7781,7 +7783,7 @@
         <v>13</v>
       </c>
       <c r="B255" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C255">
         <v>13</v>
@@ -7810,7 +7812,7 @@
         <v>13</v>
       </c>
       <c r="B256" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C256">
         <v>13</v>
@@ -8100,7 +8102,7 @@
         <v>13</v>
       </c>
       <c r="B266" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C266">
         <v>13</v>
@@ -8158,7 +8160,7 @@
         <v>13</v>
       </c>
       <c r="B268" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C268">
         <v>13</v>
@@ -8288,7 +8290,7 @@
         <v>14</v>
       </c>
       <c r="B273" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C273">
         <v>14</v>
@@ -8317,7 +8319,7 @@
         <v>14</v>
       </c>
       <c r="B274" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C274">
         <v>14</v>
@@ -8578,7 +8580,7 @@
         <v>14</v>
       </c>
       <c r="B283" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C283">
         <v>14</v>
@@ -8636,7 +8638,7 @@
         <v>14</v>
       </c>
       <c r="B285" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C285">
         <v>14</v>
@@ -8720,7 +8722,7 @@
         <v>15</v>
       </c>
       <c r="B288" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C288">
         <v>15</v>
@@ -8752,7 +8754,7 @@
         <v>15</v>
       </c>
       <c r="B289" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C289">
         <v>15</v>
@@ -8781,7 +8783,7 @@
         <v>15</v>
       </c>
       <c r="B290" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C290">
         <v>15</v>
@@ -9013,7 +9015,7 @@
         <v>15</v>
       </c>
       <c r="B298" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C298">
         <v>15</v>
@@ -9042,7 +9044,7 @@
         <v>15</v>
       </c>
       <c r="B299" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C299">
         <v>15</v>
@@ -9063,6 +9065,3343 @@
         <v>0</v>
       </c>
       <c r="J299">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="300" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A300">
+        <v>16</v>
+      </c>
+      <c r="B300" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C300">
+        <v>16</v>
+      </c>
+      <c r="D300" t="s">
+        <v>26</v>
+      </c>
+      <c r="E300">
+        <v>49</v>
+      </c>
+      <c r="F300">
+        <v>1</v>
+      </c>
+      <c r="G300">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="301" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A301">
+        <v>16</v>
+      </c>
+      <c r="B301" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C301">
+        <v>16</v>
+      </c>
+      <c r="D301" t="s">
+        <v>49</v>
+      </c>
+      <c r="E301">
+        <v>33</v>
+      </c>
+      <c r="F301">
+        <v>1</v>
+      </c>
+      <c r="G301">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="302" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A302">
+        <v>16</v>
+      </c>
+      <c r="B302" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C302">
+        <v>16</v>
+      </c>
+      <c r="D302" t="s">
+        <v>49</v>
+      </c>
+      <c r="E302">
+        <v>65</v>
+      </c>
+      <c r="F302">
+        <v>1</v>
+      </c>
+      <c r="G302">
+        <v>11</v>
+      </c>
+      <c r="H302">
+        <v>70</v>
+      </c>
+      <c r="I302">
+        <v>1</v>
+      </c>
+      <c r="J302">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="303" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A303">
+        <v>16</v>
+      </c>
+      <c r="B303" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C303">
+        <v>16</v>
+      </c>
+      <c r="D303" t="s">
+        <v>49</v>
+      </c>
+      <c r="E303">
+        <v>86</v>
+      </c>
+      <c r="F303">
+        <v>1</v>
+      </c>
+      <c r="G303">
+        <v>11</v>
+      </c>
+      <c r="H303">
+        <v>12</v>
+      </c>
+      <c r="I303">
+        <v>0</v>
+      </c>
+      <c r="J303">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="304" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A304">
+        <v>16</v>
+      </c>
+      <c r="B304" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C304">
+        <v>16</v>
+      </c>
+      <c r="D304" t="s">
+        <v>51</v>
+      </c>
+      <c r="F304">
+        <v>1</v>
+      </c>
+      <c r="G304">
+        <v>11</v>
+      </c>
+      <c r="H304">
+        <v>90</v>
+      </c>
+      <c r="I304">
+        <v>1</v>
+      </c>
+      <c r="J304">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="305" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A305">
+        <v>16</v>
+      </c>
+      <c r="B305" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C305">
+        <v>16</v>
+      </c>
+      <c r="D305" t="s">
+        <v>51</v>
+      </c>
+      <c r="F305">
+        <v>1</v>
+      </c>
+      <c r="G305">
+        <v>11</v>
+      </c>
+      <c r="H305">
+        <v>55</v>
+      </c>
+      <c r="I305">
+        <v>1</v>
+      </c>
+      <c r="J305">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="306" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A306">
+        <v>16</v>
+      </c>
+      <c r="B306" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C306">
+        <v>16</v>
+      </c>
+      <c r="D306" t="s">
+        <v>51</v>
+      </c>
+      <c r="F306">
+        <v>1</v>
+      </c>
+      <c r="G306">
+        <v>11</v>
+      </c>
+      <c r="H306">
+        <v>90</v>
+      </c>
+      <c r="I306">
+        <v>1</v>
+      </c>
+      <c r="J306">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="307" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A307">
+        <v>16</v>
+      </c>
+      <c r="B307" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C307">
+        <v>16</v>
+      </c>
+      <c r="D307" t="s">
+        <v>51</v>
+      </c>
+      <c r="F307">
+        <v>1</v>
+      </c>
+      <c r="G307">
+        <v>11</v>
+      </c>
+      <c r="H307">
+        <v>90</v>
+      </c>
+      <c r="I307">
+        <v>1</v>
+      </c>
+      <c r="J307">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="308" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A308">
+        <v>16</v>
+      </c>
+      <c r="B308" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C308">
+        <v>16</v>
+      </c>
+      <c r="D308" t="s">
+        <v>51</v>
+      </c>
+      <c r="F308">
+        <v>1</v>
+      </c>
+      <c r="G308">
+        <v>11</v>
+      </c>
+      <c r="H308">
+        <v>90</v>
+      </c>
+      <c r="I308">
+        <v>1</v>
+      </c>
+      <c r="J308">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="309" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A309">
+        <v>16</v>
+      </c>
+      <c r="B309" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C309">
+        <v>16</v>
+      </c>
+      <c r="D309" t="s">
+        <v>51</v>
+      </c>
+      <c r="F309">
+        <v>1</v>
+      </c>
+      <c r="G309">
+        <v>11</v>
+      </c>
+      <c r="H309">
+        <v>78</v>
+      </c>
+      <c r="I309">
+        <v>1</v>
+      </c>
+      <c r="J309">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="310" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A310">
+        <v>16</v>
+      </c>
+      <c r="B310" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C310">
+        <v>16</v>
+      </c>
+      <c r="D310" t="s">
+        <v>51</v>
+      </c>
+      <c r="F310">
+        <v>1</v>
+      </c>
+      <c r="G310">
+        <v>11</v>
+      </c>
+      <c r="H310">
+        <v>78</v>
+      </c>
+      <c r="I310">
+        <v>1</v>
+      </c>
+      <c r="J310">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="311" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A311">
+        <v>16</v>
+      </c>
+      <c r="B311" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C311">
+        <v>16</v>
+      </c>
+      <c r="D311" t="s">
+        <v>51</v>
+      </c>
+      <c r="F311">
+        <v>1</v>
+      </c>
+      <c r="G311">
+        <v>11</v>
+      </c>
+      <c r="H311">
+        <v>90</v>
+      </c>
+      <c r="I311">
+        <v>1</v>
+      </c>
+      <c r="J311">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="312" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A312">
+        <v>16</v>
+      </c>
+      <c r="B312" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C312">
+        <v>16</v>
+      </c>
+      <c r="D312" t="s">
+        <v>51</v>
+      </c>
+      <c r="F312">
+        <v>1</v>
+      </c>
+      <c r="G312">
+        <v>11</v>
+      </c>
+      <c r="H312">
+        <v>78</v>
+      </c>
+      <c r="I312">
+        <v>1</v>
+      </c>
+      <c r="J312">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="313" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A313">
+        <v>16</v>
+      </c>
+      <c r="B313" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C313">
+        <v>16</v>
+      </c>
+      <c r="D313" t="s">
+        <v>51</v>
+      </c>
+      <c r="F313">
+        <v>1</v>
+      </c>
+      <c r="G313">
+        <v>11</v>
+      </c>
+      <c r="H313">
+        <v>90</v>
+      </c>
+      <c r="I313">
+        <v>1</v>
+      </c>
+      <c r="J313">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="314" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A314">
+        <v>16</v>
+      </c>
+      <c r="B314" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C314">
+        <v>16</v>
+      </c>
+      <c r="D314" t="s">
+        <v>51</v>
+      </c>
+      <c r="F314">
+        <v>1</v>
+      </c>
+      <c r="G314">
+        <v>11</v>
+      </c>
+      <c r="H314">
+        <v>12</v>
+      </c>
+      <c r="I314">
+        <v>0</v>
+      </c>
+      <c r="J314">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="315" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A315">
+        <v>16</v>
+      </c>
+      <c r="B315" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C315">
+        <v>16</v>
+      </c>
+      <c r="D315" t="s">
+        <v>51</v>
+      </c>
+      <c r="F315">
+        <v>1</v>
+      </c>
+      <c r="G315">
+        <v>11</v>
+      </c>
+      <c r="H315">
+        <v>12</v>
+      </c>
+      <c r="I315">
+        <v>0</v>
+      </c>
+      <c r="J315">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="316" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A316">
+        <v>16</v>
+      </c>
+      <c r="B316" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C316">
+        <v>16</v>
+      </c>
+      <c r="D316" t="s">
+        <v>51</v>
+      </c>
+      <c r="F316">
+        <v>1</v>
+      </c>
+      <c r="G316">
+        <v>11</v>
+      </c>
+      <c r="H316">
+        <v>20</v>
+      </c>
+      <c r="I316">
+        <v>0</v>
+      </c>
+      <c r="J316">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="317" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A317">
+        <v>16</v>
+      </c>
+      <c r="B317" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C317">
+        <v>16</v>
+      </c>
+      <c r="D317" t="s">
+        <v>51</v>
+      </c>
+      <c r="F317">
+        <v>1</v>
+      </c>
+      <c r="G317">
+        <v>11</v>
+      </c>
+      <c r="H317">
+        <v>35</v>
+      </c>
+      <c r="I317">
+        <v>0</v>
+      </c>
+      <c r="J317">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="318" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A318">
+        <v>17</v>
+      </c>
+      <c r="B318" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C318">
+        <v>17</v>
+      </c>
+      <c r="D318" t="s">
+        <v>26</v>
+      </c>
+      <c r="E318">
+        <v>45</v>
+      </c>
+      <c r="F318">
+        <v>7</v>
+      </c>
+      <c r="G318">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="319" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A319">
+        <v>17</v>
+      </c>
+      <c r="B319" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C319">
+        <v>17</v>
+      </c>
+      <c r="D319" t="s">
+        <v>26</v>
+      </c>
+      <c r="E319">
+        <v>66</v>
+      </c>
+      <c r="F319">
+        <v>7</v>
+      </c>
+      <c r="G319">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="320" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A320">
+        <v>17</v>
+      </c>
+      <c r="B320" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C320">
+        <v>17</v>
+      </c>
+      <c r="D320" t="s">
+        <v>26</v>
+      </c>
+      <c r="E320">
+        <v>79</v>
+      </c>
+      <c r="F320">
+        <v>7</v>
+      </c>
+      <c r="G320">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="321" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A321">
+        <v>17</v>
+      </c>
+      <c r="B321" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C321">
+        <v>17</v>
+      </c>
+      <c r="D321" t="s">
+        <v>49</v>
+      </c>
+      <c r="E321">
+        <v>38</v>
+      </c>
+      <c r="F321">
+        <v>7</v>
+      </c>
+      <c r="G321">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="322" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A322">
+        <v>17</v>
+      </c>
+      <c r="B322" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C322">
+        <v>17</v>
+      </c>
+      <c r="D322" t="s">
+        <v>26</v>
+      </c>
+      <c r="E322">
+        <v>30</v>
+      </c>
+      <c r="F322">
+        <v>7</v>
+      </c>
+      <c r="G322">
+        <v>1</v>
+      </c>
+      <c r="H322">
+        <v>90</v>
+      </c>
+      <c r="I322">
+        <v>1</v>
+      </c>
+      <c r="J322">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="323" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A323">
+        <v>17</v>
+      </c>
+      <c r="B323" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C323">
+        <v>17</v>
+      </c>
+      <c r="D323" t="s">
+        <v>26</v>
+      </c>
+      <c r="E323">
+        <v>32</v>
+      </c>
+      <c r="F323">
+        <v>7</v>
+      </c>
+      <c r="G323">
+        <v>1</v>
+      </c>
+      <c r="H323">
+        <v>90</v>
+      </c>
+      <c r="I323">
+        <v>1</v>
+      </c>
+      <c r="J323">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="324" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A324">
+        <v>17</v>
+      </c>
+      <c r="B324" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C324">
+        <v>17</v>
+      </c>
+      <c r="D324" t="s">
+        <v>26</v>
+      </c>
+      <c r="E324">
+        <v>52</v>
+      </c>
+      <c r="F324">
+        <v>7</v>
+      </c>
+      <c r="G324">
+        <v>1</v>
+      </c>
+      <c r="H324">
+        <v>90</v>
+      </c>
+      <c r="I324">
+        <v>1</v>
+      </c>
+      <c r="J324">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="325" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A325">
+        <v>17</v>
+      </c>
+      <c r="B325" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C325">
+        <v>17</v>
+      </c>
+      <c r="D325" t="s">
+        <v>26</v>
+      </c>
+      <c r="E325">
+        <v>60</v>
+      </c>
+      <c r="F325">
+        <v>7</v>
+      </c>
+      <c r="G325">
+        <v>1</v>
+      </c>
+      <c r="H325">
+        <v>90</v>
+      </c>
+      <c r="I325">
+        <v>1</v>
+      </c>
+      <c r="J325">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="326" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A326">
+        <v>17</v>
+      </c>
+      <c r="B326" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C326">
+        <v>17</v>
+      </c>
+      <c r="D326" t="s">
+        <v>49</v>
+      </c>
+      <c r="E326">
+        <v>1</v>
+      </c>
+      <c r="F326">
+        <v>7</v>
+      </c>
+      <c r="G326">
+        <v>1</v>
+      </c>
+      <c r="H326">
+        <v>90</v>
+      </c>
+      <c r="I326">
+        <v>1</v>
+      </c>
+      <c r="J326">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="327" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A327">
+        <v>17</v>
+      </c>
+      <c r="B327" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C327">
+        <v>17</v>
+      </c>
+      <c r="D327" t="s">
+        <v>49</v>
+      </c>
+      <c r="E327">
+        <v>44</v>
+      </c>
+      <c r="F327">
+        <v>7</v>
+      </c>
+      <c r="G327">
+        <v>1</v>
+      </c>
+      <c r="H327">
+        <v>62</v>
+      </c>
+      <c r="I327">
+        <v>1</v>
+      </c>
+      <c r="J327">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="328" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A328">
+        <v>17</v>
+      </c>
+      <c r="B328" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C328">
+        <v>17</v>
+      </c>
+      <c r="D328" t="s">
+        <v>51</v>
+      </c>
+      <c r="F328">
+        <v>7</v>
+      </c>
+      <c r="G328">
+        <v>1</v>
+      </c>
+      <c r="H328">
+        <v>90</v>
+      </c>
+      <c r="I328">
+        <v>1</v>
+      </c>
+      <c r="J328">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="329" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A329">
+        <v>17</v>
+      </c>
+      <c r="B329" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C329">
+        <v>17</v>
+      </c>
+      <c r="D329" t="s">
+        <v>51</v>
+      </c>
+      <c r="F329">
+        <v>7</v>
+      </c>
+      <c r="G329">
+        <v>1</v>
+      </c>
+      <c r="H329">
+        <v>90</v>
+      </c>
+      <c r="I329">
+        <v>1</v>
+      </c>
+      <c r="J329">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="330" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A330">
+        <v>17</v>
+      </c>
+      <c r="B330" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C330">
+        <v>17</v>
+      </c>
+      <c r="D330" t="s">
+        <v>51</v>
+      </c>
+      <c r="F330">
+        <v>7</v>
+      </c>
+      <c r="G330">
+        <v>1</v>
+      </c>
+      <c r="H330">
+        <v>90</v>
+      </c>
+      <c r="I330">
+        <v>1</v>
+      </c>
+      <c r="J330">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="331" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A331">
+        <v>17</v>
+      </c>
+      <c r="B331" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C331">
+        <v>17</v>
+      </c>
+      <c r="D331" t="s">
+        <v>51</v>
+      </c>
+      <c r="F331">
+        <v>7</v>
+      </c>
+      <c r="G331">
+        <v>1</v>
+      </c>
+      <c r="H331">
+        <v>49</v>
+      </c>
+      <c r="I331">
+        <v>1</v>
+      </c>
+      <c r="J331">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="332" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A332">
+        <v>17</v>
+      </c>
+      <c r="B332" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C332">
+        <v>17</v>
+      </c>
+      <c r="D332" t="s">
+        <v>51</v>
+      </c>
+      <c r="F332">
+        <v>7</v>
+      </c>
+      <c r="G332">
+        <v>1</v>
+      </c>
+      <c r="H332">
+        <v>82</v>
+      </c>
+      <c r="I332">
+        <v>1</v>
+      </c>
+      <c r="J332">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="333" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A333">
+        <v>17</v>
+      </c>
+      <c r="B333" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C333">
+        <v>17</v>
+      </c>
+      <c r="D333" t="s">
+        <v>51</v>
+      </c>
+      <c r="F333">
+        <v>7</v>
+      </c>
+      <c r="G333">
+        <v>1</v>
+      </c>
+      <c r="H333">
+        <v>90</v>
+      </c>
+      <c r="I333">
+        <v>1</v>
+      </c>
+      <c r="J333">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="334" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A334">
+        <v>17</v>
+      </c>
+      <c r="B334" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C334">
+        <v>17</v>
+      </c>
+      <c r="D334" t="s">
+        <v>51</v>
+      </c>
+      <c r="F334">
+        <v>7</v>
+      </c>
+      <c r="G334">
+        <v>1</v>
+      </c>
+      <c r="H334">
+        <v>8</v>
+      </c>
+      <c r="I334">
+        <v>0</v>
+      </c>
+      <c r="J334">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="335" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A335">
+        <v>17</v>
+      </c>
+      <c r="B335" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C335">
+        <v>17</v>
+      </c>
+      <c r="D335" t="s">
+        <v>51</v>
+      </c>
+      <c r="F335">
+        <v>7</v>
+      </c>
+      <c r="G335">
+        <v>1</v>
+      </c>
+      <c r="H335">
+        <v>28</v>
+      </c>
+      <c r="I335">
+        <v>0</v>
+      </c>
+      <c r="J335">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="336" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A336">
+        <v>17</v>
+      </c>
+      <c r="B336" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C336">
+        <v>17</v>
+      </c>
+      <c r="D336" t="s">
+        <v>51</v>
+      </c>
+      <c r="F336">
+        <v>7</v>
+      </c>
+      <c r="G336">
+        <v>1</v>
+      </c>
+      <c r="H336">
+        <v>41</v>
+      </c>
+      <c r="I336">
+        <v>0</v>
+      </c>
+      <c r="J336">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="337" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A337">
+        <v>18</v>
+      </c>
+      <c r="B337" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C337">
+        <v>18</v>
+      </c>
+      <c r="D337" t="s">
+        <v>26</v>
+      </c>
+      <c r="E337">
+        <v>43</v>
+      </c>
+      <c r="F337">
+        <v>2</v>
+      </c>
+      <c r="G337">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="338" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A338">
+        <v>18</v>
+      </c>
+      <c r="B338" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C338">
+        <v>18</v>
+      </c>
+      <c r="D338" t="s">
+        <v>26</v>
+      </c>
+      <c r="E338">
+        <v>48</v>
+      </c>
+      <c r="F338">
+        <v>2</v>
+      </c>
+      <c r="G338">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="339" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A339">
+        <v>18</v>
+      </c>
+      <c r="B339" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C339">
+        <v>18</v>
+      </c>
+      <c r="D339" t="s">
+        <v>26</v>
+      </c>
+      <c r="E339">
+        <v>69</v>
+      </c>
+      <c r="F339">
+        <v>2</v>
+      </c>
+      <c r="G339">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="340" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A340">
+        <v>18</v>
+      </c>
+      <c r="B340" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C340">
+        <v>18</v>
+      </c>
+      <c r="D340" t="s">
+        <v>26</v>
+      </c>
+      <c r="E340">
+        <v>87</v>
+      </c>
+      <c r="F340">
+        <v>2</v>
+      </c>
+      <c r="G340">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="341" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A341">
+        <v>18</v>
+      </c>
+      <c r="B341" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C341">
+        <v>18</v>
+      </c>
+      <c r="D341" t="s">
+        <v>26</v>
+      </c>
+      <c r="E341">
+        <v>92</v>
+      </c>
+      <c r="F341">
+        <v>2</v>
+      </c>
+      <c r="G341">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="342" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A342">
+        <v>18</v>
+      </c>
+      <c r="B342" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C342">
+        <v>18</v>
+      </c>
+      <c r="D342" t="s">
+        <v>49</v>
+      </c>
+      <c r="E342">
+        <v>44</v>
+      </c>
+      <c r="F342">
+        <v>2</v>
+      </c>
+      <c r="G342">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="343" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A343">
+        <v>18</v>
+      </c>
+      <c r="B343" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C343">
+        <v>18</v>
+      </c>
+      <c r="D343" t="s">
+        <v>49</v>
+      </c>
+      <c r="E343">
+        <v>49</v>
+      </c>
+      <c r="F343">
+        <v>2</v>
+      </c>
+      <c r="G343">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="344" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A344">
+        <v>18</v>
+      </c>
+      <c r="B344" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C344">
+        <v>18</v>
+      </c>
+      <c r="D344" t="s">
+        <v>26</v>
+      </c>
+      <c r="E344">
+        <v>3</v>
+      </c>
+      <c r="F344">
+        <v>2</v>
+      </c>
+      <c r="G344">
+        <v>1</v>
+      </c>
+      <c r="H344">
+        <v>90</v>
+      </c>
+      <c r="I344">
+        <v>1</v>
+      </c>
+      <c r="J344">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="345" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A345">
+        <v>18</v>
+      </c>
+      <c r="B345" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C345">
+        <v>18</v>
+      </c>
+      <c r="D345" t="s">
+        <v>49</v>
+      </c>
+      <c r="E345">
+        <v>17</v>
+      </c>
+      <c r="F345">
+        <v>2</v>
+      </c>
+      <c r="G345">
+        <v>1</v>
+      </c>
+      <c r="H345">
+        <v>90</v>
+      </c>
+      <c r="I345">
+        <v>1</v>
+      </c>
+      <c r="J345">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="346" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A346">
+        <v>18</v>
+      </c>
+      <c r="B346" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C346">
+        <v>18</v>
+      </c>
+      <c r="D346" t="s">
+        <v>49</v>
+      </c>
+      <c r="E346">
+        <v>45</v>
+      </c>
+      <c r="F346">
+        <v>2</v>
+      </c>
+      <c r="G346">
+        <v>1</v>
+      </c>
+      <c r="H346">
+        <v>90</v>
+      </c>
+      <c r="I346">
+        <v>1</v>
+      </c>
+      <c r="J346">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="347" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A347">
+        <v>18</v>
+      </c>
+      <c r="B347" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C347">
+        <v>18</v>
+      </c>
+      <c r="D347" t="s">
+        <v>51</v>
+      </c>
+      <c r="F347">
+        <v>2</v>
+      </c>
+      <c r="G347">
+        <v>1</v>
+      </c>
+      <c r="H347">
+        <v>90</v>
+      </c>
+      <c r="I347">
+        <v>1</v>
+      </c>
+      <c r="J347">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="348" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A348">
+        <v>18</v>
+      </c>
+      <c r="B348" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C348">
+        <v>18</v>
+      </c>
+      <c r="D348" t="s">
+        <v>51</v>
+      </c>
+      <c r="F348">
+        <v>2</v>
+      </c>
+      <c r="G348">
+        <v>1</v>
+      </c>
+      <c r="H348">
+        <v>90</v>
+      </c>
+      <c r="I348">
+        <v>1</v>
+      </c>
+      <c r="J348">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="349" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A349">
+        <v>18</v>
+      </c>
+      <c r="B349" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C349">
+        <v>18</v>
+      </c>
+      <c r="D349" t="s">
+        <v>51</v>
+      </c>
+      <c r="F349">
+        <v>2</v>
+      </c>
+      <c r="G349">
+        <v>1</v>
+      </c>
+      <c r="H349">
+        <v>90</v>
+      </c>
+      <c r="I349">
+        <v>1</v>
+      </c>
+      <c r="J349">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="350" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A350">
+        <v>18</v>
+      </c>
+      <c r="B350" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C350">
+        <v>18</v>
+      </c>
+      <c r="D350" t="s">
+        <v>51</v>
+      </c>
+      <c r="F350">
+        <v>2</v>
+      </c>
+      <c r="G350">
+        <v>1</v>
+      </c>
+      <c r="H350">
+        <v>75</v>
+      </c>
+      <c r="I350">
+        <v>1</v>
+      </c>
+      <c r="J350">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="351" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A351">
+        <v>18</v>
+      </c>
+      <c r="B351" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C351">
+        <v>18</v>
+      </c>
+      <c r="D351" t="s">
+        <v>51</v>
+      </c>
+      <c r="F351">
+        <v>2</v>
+      </c>
+      <c r="G351">
+        <v>1</v>
+      </c>
+      <c r="H351">
+        <v>90</v>
+      </c>
+      <c r="I351">
+        <v>1</v>
+      </c>
+      <c r="J351">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="352" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A352">
+        <v>18</v>
+      </c>
+      <c r="B352" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C352">
+        <v>18</v>
+      </c>
+      <c r="D352" t="s">
+        <v>51</v>
+      </c>
+      <c r="F352">
+        <v>2</v>
+      </c>
+      <c r="G352">
+        <v>1</v>
+      </c>
+      <c r="H352">
+        <v>90</v>
+      </c>
+      <c r="I352">
+        <v>1</v>
+      </c>
+      <c r="J352">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="353" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A353">
+        <v>18</v>
+      </c>
+      <c r="B353" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C353">
+        <v>18</v>
+      </c>
+      <c r="D353" t="s">
+        <v>51</v>
+      </c>
+      <c r="F353">
+        <v>2</v>
+      </c>
+      <c r="G353">
+        <v>1</v>
+      </c>
+      <c r="H353">
+        <v>75</v>
+      </c>
+      <c r="I353">
+        <v>1</v>
+      </c>
+      <c r="J353">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="354" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A354">
+        <v>18</v>
+      </c>
+      <c r="B354" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C354">
+        <v>18</v>
+      </c>
+      <c r="D354" t="s">
+        <v>51</v>
+      </c>
+      <c r="F354">
+        <v>2</v>
+      </c>
+      <c r="G354">
+        <v>1</v>
+      </c>
+      <c r="H354">
+        <v>90</v>
+      </c>
+      <c r="I354">
+        <v>1</v>
+      </c>
+      <c r="J354">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="355" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A355">
+        <v>18</v>
+      </c>
+      <c r="B355" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C355">
+        <v>18</v>
+      </c>
+      <c r="D355" t="s">
+        <v>51</v>
+      </c>
+      <c r="F355">
+        <v>2</v>
+      </c>
+      <c r="G355">
+        <v>1</v>
+      </c>
+      <c r="H355">
+        <v>15</v>
+      </c>
+      <c r="I355">
+        <v>0</v>
+      </c>
+      <c r="J355">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="356" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A356">
+        <v>18</v>
+      </c>
+      <c r="B356" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C356">
+        <v>18</v>
+      </c>
+      <c r="D356" t="s">
+        <v>51</v>
+      </c>
+      <c r="F356">
+        <v>2</v>
+      </c>
+      <c r="G356">
+        <v>1</v>
+      </c>
+      <c r="H356">
+        <v>15</v>
+      </c>
+      <c r="I356">
+        <v>0</v>
+      </c>
+      <c r="J356">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="357" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A357">
+        <v>19</v>
+      </c>
+      <c r="B357" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C357">
+        <v>19</v>
+      </c>
+      <c r="D357" t="s">
+        <v>26</v>
+      </c>
+      <c r="E357">
+        <v>81</v>
+      </c>
+      <c r="F357">
+        <v>1</v>
+      </c>
+      <c r="G357">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="358" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A358">
+        <v>19</v>
+      </c>
+      <c r="B358" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C358">
+        <v>19</v>
+      </c>
+      <c r="D358" t="s">
+        <v>49</v>
+      </c>
+      <c r="E358">
+        <v>57</v>
+      </c>
+      <c r="F358">
+        <v>1</v>
+      </c>
+      <c r="G358">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="359" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A359">
+        <v>19</v>
+      </c>
+      <c r="B359" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C359">
+        <v>19</v>
+      </c>
+      <c r="D359" t="s">
+        <v>49</v>
+      </c>
+      <c r="E359">
+        <v>75</v>
+      </c>
+      <c r="F359">
+        <v>1</v>
+      </c>
+      <c r="G359">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="360" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A360">
+        <v>19</v>
+      </c>
+      <c r="B360" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C360">
+        <v>19</v>
+      </c>
+      <c r="D360" t="s">
+        <v>49</v>
+      </c>
+      <c r="E360">
+        <v>76</v>
+      </c>
+      <c r="F360">
+        <v>1</v>
+      </c>
+      <c r="G360">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="361" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A361">
+        <v>19</v>
+      </c>
+      <c r="B361" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C361">
+        <v>19</v>
+      </c>
+      <c r="D361" t="s">
+        <v>49</v>
+      </c>
+      <c r="E361">
+        <v>90</v>
+      </c>
+      <c r="F361">
+        <v>1</v>
+      </c>
+      <c r="G361">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="362" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A362">
+        <v>19</v>
+      </c>
+      <c r="B362" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C362">
+        <v>19</v>
+      </c>
+      <c r="D362" t="s">
+        <v>26</v>
+      </c>
+      <c r="E362">
+        <v>3</v>
+      </c>
+      <c r="F362">
+        <v>1</v>
+      </c>
+      <c r="G362">
+        <v>15</v>
+      </c>
+      <c r="H362">
+        <v>89</v>
+      </c>
+      <c r="I362">
+        <v>1</v>
+      </c>
+      <c r="J362">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="363" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A363">
+        <v>19</v>
+      </c>
+      <c r="B363" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C363">
+        <v>19</v>
+      </c>
+      <c r="D363" t="s">
+        <v>26</v>
+      </c>
+      <c r="E363">
+        <v>34</v>
+      </c>
+      <c r="F363">
+        <v>1</v>
+      </c>
+      <c r="G363">
+        <v>15</v>
+      </c>
+      <c r="H363">
+        <v>90</v>
+      </c>
+      <c r="I363">
+        <v>1</v>
+      </c>
+      <c r="J363">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="364" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A364">
+        <v>19</v>
+      </c>
+      <c r="B364" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C364">
+        <v>19</v>
+      </c>
+      <c r="D364" t="s">
+        <v>49</v>
+      </c>
+      <c r="E364">
+        <v>83</v>
+      </c>
+      <c r="F364">
+        <v>1</v>
+      </c>
+      <c r="G364">
+        <v>15</v>
+      </c>
+      <c r="H364">
+        <v>90</v>
+      </c>
+      <c r="I364">
+        <v>1</v>
+      </c>
+      <c r="J364">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="365" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A365">
+        <v>19</v>
+      </c>
+      <c r="B365" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C365">
+        <v>19</v>
+      </c>
+      <c r="D365" t="s">
+        <v>51</v>
+      </c>
+      <c r="F365">
+        <v>1</v>
+      </c>
+      <c r="G365">
+        <v>15</v>
+      </c>
+      <c r="H365">
+        <v>65</v>
+      </c>
+      <c r="I365">
+        <v>1</v>
+      </c>
+      <c r="J365">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="366" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A366">
+        <v>19</v>
+      </c>
+      <c r="B366" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C366">
+        <v>19</v>
+      </c>
+      <c r="D366" t="s">
+        <v>51</v>
+      </c>
+      <c r="F366">
+        <v>1</v>
+      </c>
+      <c r="G366">
+        <v>15</v>
+      </c>
+      <c r="H366">
+        <v>90</v>
+      </c>
+      <c r="I366">
+        <v>1</v>
+      </c>
+      <c r="J366">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="367" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A367">
+        <v>19</v>
+      </c>
+      <c r="B367" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C367">
+        <v>19</v>
+      </c>
+      <c r="D367" t="s">
+        <v>51</v>
+      </c>
+      <c r="F367">
+        <v>1</v>
+      </c>
+      <c r="G367">
+        <v>15</v>
+      </c>
+      <c r="H367">
+        <v>90</v>
+      </c>
+      <c r="I367">
+        <v>1</v>
+      </c>
+      <c r="J367">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="368" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A368">
+        <v>19</v>
+      </c>
+      <c r="B368" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C368">
+        <v>19</v>
+      </c>
+      <c r="D368" t="s">
+        <v>51</v>
+      </c>
+      <c r="F368">
+        <v>1</v>
+      </c>
+      <c r="G368">
+        <v>15</v>
+      </c>
+      <c r="H368">
+        <v>45</v>
+      </c>
+      <c r="I368">
+        <v>1</v>
+      </c>
+      <c r="J368">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="369" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A369">
+        <v>19</v>
+      </c>
+      <c r="B369" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C369">
+        <v>19</v>
+      </c>
+      <c r="D369" t="s">
+        <v>51</v>
+      </c>
+      <c r="F369">
+        <v>1</v>
+      </c>
+      <c r="G369">
+        <v>15</v>
+      </c>
+      <c r="H369">
+        <v>90</v>
+      </c>
+      <c r="I369">
+        <v>1</v>
+      </c>
+      <c r="J369">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="370" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A370">
+        <v>19</v>
+      </c>
+      <c r="B370" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C370">
+        <v>19</v>
+      </c>
+      <c r="D370" t="s">
+        <v>51</v>
+      </c>
+      <c r="F370">
+        <v>1</v>
+      </c>
+      <c r="G370">
+        <v>15</v>
+      </c>
+      <c r="H370">
+        <v>90</v>
+      </c>
+      <c r="I370">
+        <v>1</v>
+      </c>
+      <c r="J370">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="371" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A371">
+        <v>19</v>
+      </c>
+      <c r="B371" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C371">
+        <v>19</v>
+      </c>
+      <c r="D371" t="s">
+        <v>51</v>
+      </c>
+      <c r="F371">
+        <v>1</v>
+      </c>
+      <c r="G371">
+        <v>15</v>
+      </c>
+      <c r="H371">
+        <v>90</v>
+      </c>
+      <c r="I371">
+        <v>1</v>
+      </c>
+      <c r="J371">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="372" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A372">
+        <v>19</v>
+      </c>
+      <c r="B372" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C372">
+        <v>19</v>
+      </c>
+      <c r="D372" t="s">
+        <v>51</v>
+      </c>
+      <c r="F372">
+        <v>1</v>
+      </c>
+      <c r="G372">
+        <v>15</v>
+      </c>
+      <c r="H372">
+        <v>25</v>
+      </c>
+      <c r="I372">
+        <v>0</v>
+      </c>
+      <c r="J372">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="373" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A373">
+        <v>19</v>
+      </c>
+      <c r="B373" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C373">
+        <v>19</v>
+      </c>
+      <c r="D373" t="s">
+        <v>51</v>
+      </c>
+      <c r="F373">
+        <v>1</v>
+      </c>
+      <c r="G373">
+        <v>15</v>
+      </c>
+      <c r="H373">
+        <v>1</v>
+      </c>
+      <c r="I373">
+        <v>0</v>
+      </c>
+      <c r="J373">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="374" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A374">
+        <v>19</v>
+      </c>
+      <c r="B374" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C374">
+        <v>19</v>
+      </c>
+      <c r="D374" t="s">
+        <v>51</v>
+      </c>
+      <c r="F374">
+        <v>1</v>
+      </c>
+      <c r="G374">
+        <v>15</v>
+      </c>
+      <c r="H374">
+        <v>45</v>
+      </c>
+      <c r="I374">
+        <v>0</v>
+      </c>
+      <c r="J374">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="375" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A375">
+        <v>20</v>
+      </c>
+      <c r="B375" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C375">
+        <v>20</v>
+      </c>
+      <c r="D375" t="s">
+        <v>26</v>
+      </c>
+      <c r="E375">
+        <v>20</v>
+      </c>
+      <c r="F375">
+        <v>14</v>
+      </c>
+      <c r="G375">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="376" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A376">
+        <v>20</v>
+      </c>
+      <c r="B376" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C376">
+        <v>20</v>
+      </c>
+      <c r="D376" t="s">
+        <v>26</v>
+      </c>
+      <c r="E376">
+        <v>90</v>
+      </c>
+      <c r="F376">
+        <v>14</v>
+      </c>
+      <c r="G376">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="377" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A377">
+        <v>20</v>
+      </c>
+      <c r="B377" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C377">
+        <v>20</v>
+      </c>
+      <c r="D377" t="s">
+        <v>49</v>
+      </c>
+      <c r="E377">
+        <v>68</v>
+      </c>
+      <c r="F377">
+        <v>14</v>
+      </c>
+      <c r="G377">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="378" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A378">
+        <v>20</v>
+      </c>
+      <c r="B378" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C378">
+        <v>20</v>
+      </c>
+      <c r="D378" t="s">
+        <v>49</v>
+      </c>
+      <c r="E378">
+        <v>72</v>
+      </c>
+      <c r="F378">
+        <v>14</v>
+      </c>
+      <c r="G378">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="379" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A379">
+        <v>20</v>
+      </c>
+      <c r="B379" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C379">
+        <v>20</v>
+      </c>
+      <c r="D379" t="s">
+        <v>49</v>
+      </c>
+      <c r="E379">
+        <v>90</v>
+      </c>
+      <c r="F379">
+        <v>14</v>
+      </c>
+      <c r="G379">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="380" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A380">
+        <v>20</v>
+      </c>
+      <c r="B380" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C380">
+        <v>20</v>
+      </c>
+      <c r="D380" t="s">
+        <v>49</v>
+      </c>
+      <c r="E380">
+        <v>90</v>
+      </c>
+      <c r="F380">
+        <v>14</v>
+      </c>
+      <c r="G380">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="381" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A381">
+        <v>20</v>
+      </c>
+      <c r="B381" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C381">
+        <v>20</v>
+      </c>
+      <c r="D381" t="s">
+        <v>26</v>
+      </c>
+      <c r="E381">
+        <v>78</v>
+      </c>
+      <c r="F381">
+        <v>14</v>
+      </c>
+      <c r="G381">
+        <v>1</v>
+      </c>
+      <c r="H381">
+        <v>90</v>
+      </c>
+      <c r="I381">
+        <v>1</v>
+      </c>
+      <c r="J381">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="382" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A382">
+        <v>20</v>
+      </c>
+      <c r="B382" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C382">
+        <v>20</v>
+      </c>
+      <c r="D382" t="s">
+        <v>49</v>
+      </c>
+      <c r="E382">
+        <v>68</v>
+      </c>
+      <c r="F382">
+        <v>14</v>
+      </c>
+      <c r="G382">
+        <v>1</v>
+      </c>
+      <c r="H382">
+        <v>5</v>
+      </c>
+      <c r="I382">
+        <v>0</v>
+      </c>
+      <c r="J382">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="383" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A383">
+        <v>20</v>
+      </c>
+      <c r="B383" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C383">
+        <v>20</v>
+      </c>
+      <c r="D383" t="s">
+        <v>49</v>
+      </c>
+      <c r="E383">
+        <v>78</v>
+      </c>
+      <c r="F383">
+        <v>14</v>
+      </c>
+      <c r="G383">
+        <v>1</v>
+      </c>
+      <c r="H383">
+        <v>90</v>
+      </c>
+      <c r="I383">
+        <v>1</v>
+      </c>
+      <c r="J383">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="384" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A384">
+        <v>20</v>
+      </c>
+      <c r="B384" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C384">
+        <v>20</v>
+      </c>
+      <c r="D384" t="s">
+        <v>49</v>
+      </c>
+      <c r="E384">
+        <v>78</v>
+      </c>
+      <c r="F384">
+        <v>14</v>
+      </c>
+      <c r="G384">
+        <v>1</v>
+      </c>
+      <c r="H384">
+        <v>90</v>
+      </c>
+      <c r="I384">
+        <v>1</v>
+      </c>
+      <c r="J384">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="385" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A385">
+        <v>20</v>
+      </c>
+      <c r="B385" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C385">
+        <v>20</v>
+      </c>
+      <c r="D385" t="s">
+        <v>51</v>
+      </c>
+      <c r="F385">
+        <v>14</v>
+      </c>
+      <c r="G385">
+        <v>1</v>
+      </c>
+      <c r="H385">
+        <v>90</v>
+      </c>
+      <c r="I385">
+        <v>1</v>
+      </c>
+      <c r="J385">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="386" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A386">
+        <v>20</v>
+      </c>
+      <c r="B386" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C386">
+        <v>20</v>
+      </c>
+      <c r="D386" t="s">
+        <v>51</v>
+      </c>
+      <c r="F386">
+        <v>14</v>
+      </c>
+      <c r="G386">
+        <v>1</v>
+      </c>
+      <c r="H386">
+        <v>45</v>
+      </c>
+      <c r="I386">
+        <v>1</v>
+      </c>
+      <c r="J386">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="387" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A387">
+        <v>20</v>
+      </c>
+      <c r="B387" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C387">
+        <v>20</v>
+      </c>
+      <c r="D387" t="s">
+        <v>51</v>
+      </c>
+      <c r="F387">
+        <v>14</v>
+      </c>
+      <c r="G387">
+        <v>1</v>
+      </c>
+      <c r="H387">
+        <v>90</v>
+      </c>
+      <c r="I387">
+        <v>1</v>
+      </c>
+      <c r="J387">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="388" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A388">
+        <v>20</v>
+      </c>
+      <c r="B388" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C388">
+        <v>20</v>
+      </c>
+      <c r="D388" t="s">
+        <v>51</v>
+      </c>
+      <c r="F388">
+        <v>14</v>
+      </c>
+      <c r="G388">
+        <v>1</v>
+      </c>
+      <c r="H388">
+        <v>90</v>
+      </c>
+      <c r="I388">
+        <v>1</v>
+      </c>
+      <c r="J388">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="389" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A389">
+        <v>20</v>
+      </c>
+      <c r="B389" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C389">
+        <v>20</v>
+      </c>
+      <c r="D389" t="s">
+        <v>51</v>
+      </c>
+      <c r="F389">
+        <v>14</v>
+      </c>
+      <c r="G389">
+        <v>1</v>
+      </c>
+      <c r="H389">
+        <v>85</v>
+      </c>
+      <c r="I389">
+        <v>1</v>
+      </c>
+      <c r="J389">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="390" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A390">
+        <v>20</v>
+      </c>
+      <c r="B390" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C390">
+        <v>20</v>
+      </c>
+      <c r="D390" t="s">
+        <v>51</v>
+      </c>
+      <c r="F390">
+        <v>14</v>
+      </c>
+      <c r="G390">
+        <v>1</v>
+      </c>
+      <c r="H390">
+        <v>66</v>
+      </c>
+      <c r="I390">
+        <v>1</v>
+      </c>
+      <c r="J390">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="391" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A391">
+        <v>20</v>
+      </c>
+      <c r="B391" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C391">
+        <v>20</v>
+      </c>
+      <c r="D391" t="s">
+        <v>51</v>
+      </c>
+      <c r="F391">
+        <v>14</v>
+      </c>
+      <c r="G391">
+        <v>1</v>
+      </c>
+      <c r="H391">
+        <v>90</v>
+      </c>
+      <c r="I391">
+        <v>1</v>
+      </c>
+      <c r="J391">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="392" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A392">
+        <v>20</v>
+      </c>
+      <c r="B392" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C392">
+        <v>20</v>
+      </c>
+      <c r="D392" t="s">
+        <v>51</v>
+      </c>
+      <c r="F392">
+        <v>14</v>
+      </c>
+      <c r="G392">
+        <v>1</v>
+      </c>
+      <c r="H392">
+        <v>90</v>
+      </c>
+      <c r="I392">
+        <v>1</v>
+      </c>
+      <c r="J392">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="393" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A393">
+        <v>20</v>
+      </c>
+      <c r="B393" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C393">
+        <v>20</v>
+      </c>
+      <c r="D393" t="s">
+        <v>51</v>
+      </c>
+      <c r="F393">
+        <v>14</v>
+      </c>
+      <c r="G393">
+        <v>1</v>
+      </c>
+      <c r="H393">
+        <v>90</v>
+      </c>
+      <c r="I393">
+        <v>1</v>
+      </c>
+      <c r="J393">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="394" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A394">
+        <v>20</v>
+      </c>
+      <c r="B394" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C394">
+        <v>20</v>
+      </c>
+      <c r="D394" t="s">
+        <v>51</v>
+      </c>
+      <c r="F394">
+        <v>14</v>
+      </c>
+      <c r="G394">
+        <v>1</v>
+      </c>
+      <c r="H394">
+        <v>45</v>
+      </c>
+      <c r="I394">
+        <v>0</v>
+      </c>
+      <c r="J394">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="395" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A395">
+        <v>20</v>
+      </c>
+      <c r="B395" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C395">
+        <v>20</v>
+      </c>
+      <c r="D395" t="s">
+        <v>51</v>
+      </c>
+      <c r="F395">
+        <v>14</v>
+      </c>
+      <c r="G395">
+        <v>1</v>
+      </c>
+      <c r="H395">
+        <v>24</v>
+      </c>
+      <c r="I395">
+        <v>0</v>
+      </c>
+      <c r="J395">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="396" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A396">
+        <v>21</v>
+      </c>
+      <c r="B396" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C396">
+        <v>21</v>
+      </c>
+      <c r="D396" t="s">
+        <v>26</v>
+      </c>
+      <c r="E396">
+        <v>54</v>
+      </c>
+      <c r="F396">
+        <v>1</v>
+      </c>
+      <c r="G396">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="397" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A397">
+        <v>21</v>
+      </c>
+      <c r="B397" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C397">
+        <v>21</v>
+      </c>
+      <c r="D397" t="s">
+        <v>49</v>
+      </c>
+      <c r="E397">
+        <v>53</v>
+      </c>
+      <c r="F397">
+        <v>1</v>
+      </c>
+      <c r="G397">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="398" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A398">
+        <v>21</v>
+      </c>
+      <c r="B398" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C398">
+        <v>21</v>
+      </c>
+      <c r="D398" t="s">
+        <v>49</v>
+      </c>
+      <c r="E398">
+        <v>73</v>
+      </c>
+      <c r="F398">
+        <v>1</v>
+      </c>
+      <c r="G398">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="399" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A399">
+        <v>21</v>
+      </c>
+      <c r="B399" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C399">
+        <v>21</v>
+      </c>
+      <c r="D399" t="s">
+        <v>49</v>
+      </c>
+      <c r="E399">
+        <v>85</v>
+      </c>
+      <c r="F399">
+        <v>1</v>
+      </c>
+      <c r="G399">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="400" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A400">
+        <v>21</v>
+      </c>
+      <c r="B400" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C400">
+        <v>21</v>
+      </c>
+      <c r="D400" t="s">
+        <v>49</v>
+      </c>
+      <c r="E400">
+        <v>88</v>
+      </c>
+      <c r="F400">
+        <v>1</v>
+      </c>
+      <c r="G400">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="401" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A401">
+        <v>21</v>
+      </c>
+      <c r="B401" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C401">
+        <v>21</v>
+      </c>
+      <c r="D401" t="s">
+        <v>49</v>
+      </c>
+      <c r="E401">
+        <v>92</v>
+      </c>
+      <c r="F401">
+        <v>1</v>
+      </c>
+      <c r="G401">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="402" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A402">
+        <v>21</v>
+      </c>
+      <c r="B402" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C402">
+        <v>21</v>
+      </c>
+      <c r="D402" t="s">
+        <v>49</v>
+      </c>
+      <c r="E402">
+        <v>94</v>
+      </c>
+      <c r="F402">
+        <v>1</v>
+      </c>
+      <c r="G402">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="403" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A403">
+        <v>21</v>
+      </c>
+      <c r="B403" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C403">
+        <v>21</v>
+      </c>
+      <c r="D403" t="s">
+        <v>26</v>
+      </c>
+      <c r="E403">
+        <v>7</v>
+      </c>
+      <c r="F403">
+        <v>1</v>
+      </c>
+      <c r="G403">
+        <v>6</v>
+      </c>
+      <c r="H403">
+        <v>85</v>
+      </c>
+      <c r="I403">
+        <v>1</v>
+      </c>
+      <c r="J403">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="404" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A404">
+        <v>21</v>
+      </c>
+      <c r="B404" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C404">
+        <v>21</v>
+      </c>
+      <c r="D404" t="s">
+        <v>26</v>
+      </c>
+      <c r="E404">
+        <v>21</v>
+      </c>
+      <c r="F404">
+        <v>1</v>
+      </c>
+      <c r="G404">
+        <v>6</v>
+      </c>
+      <c r="H404">
+        <v>57</v>
+      </c>
+      <c r="I404">
+        <v>1</v>
+      </c>
+      <c r="J404">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="405" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A405">
+        <v>21</v>
+      </c>
+      <c r="B405" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C405">
+        <v>21</v>
+      </c>
+      <c r="D405" t="s">
+        <v>49</v>
+      </c>
+      <c r="E405">
+        <v>78</v>
+      </c>
+      <c r="F405">
+        <v>1</v>
+      </c>
+      <c r="G405">
+        <v>6</v>
+      </c>
+      <c r="H405">
+        <v>85</v>
+      </c>
+      <c r="I405">
+        <v>1</v>
+      </c>
+      <c r="J405">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="406" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A406">
+        <v>21</v>
+      </c>
+      <c r="B406" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C406">
+        <v>21</v>
+      </c>
+      <c r="D406" t="s">
+        <v>49</v>
+      </c>
+      <c r="E406">
+        <v>76</v>
+      </c>
+      <c r="F406">
+        <v>1</v>
+      </c>
+      <c r="G406">
+        <v>6</v>
+      </c>
+      <c r="H406">
+        <v>90</v>
+      </c>
+      <c r="I406">
+        <v>1</v>
+      </c>
+      <c r="J406">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="407" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A407">
+        <v>21</v>
+      </c>
+      <c r="B407" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C407">
+        <v>21</v>
+      </c>
+      <c r="D407" t="s">
+        <v>49</v>
+      </c>
+      <c r="E407">
+        <v>83</v>
+      </c>
+      <c r="F407">
+        <v>1</v>
+      </c>
+      <c r="G407">
+        <v>6</v>
+      </c>
+      <c r="H407">
+        <v>90</v>
+      </c>
+      <c r="I407">
+        <v>1</v>
+      </c>
+      <c r="J407">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="408" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A408">
+        <v>21</v>
+      </c>
+      <c r="B408" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C408">
+        <v>21</v>
+      </c>
+      <c r="D408" t="s">
+        <v>49</v>
+      </c>
+      <c r="E408">
+        <v>92</v>
+      </c>
+      <c r="F408">
+        <v>1</v>
+      </c>
+      <c r="G408">
+        <v>6</v>
+      </c>
+      <c r="H408">
+        <v>90</v>
+      </c>
+      <c r="I408">
+        <v>1</v>
+      </c>
+      <c r="J408">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="409" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A409">
+        <v>21</v>
+      </c>
+      <c r="B409" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C409">
+        <v>21</v>
+      </c>
+      <c r="D409" t="s">
+        <v>51</v>
+      </c>
+      <c r="F409">
+        <v>1</v>
+      </c>
+      <c r="G409">
+        <v>6</v>
+      </c>
+      <c r="H409">
+        <v>90</v>
+      </c>
+      <c r="I409">
+        <v>1</v>
+      </c>
+      <c r="J409">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="410" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A410">
+        <v>21</v>
+      </c>
+      <c r="B410" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C410">
+        <v>21</v>
+      </c>
+      <c r="D410" t="s">
+        <v>51</v>
+      </c>
+      <c r="F410">
+        <v>1</v>
+      </c>
+      <c r="G410">
+        <v>6</v>
+      </c>
+      <c r="H410">
+        <v>87</v>
+      </c>
+      <c r="I410">
+        <v>1</v>
+      </c>
+      <c r="J410">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="411" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A411">
+        <v>21</v>
+      </c>
+      <c r="B411" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C411">
+        <v>21</v>
+      </c>
+      <c r="D411" t="s">
+        <v>51</v>
+      </c>
+      <c r="F411">
+        <v>1</v>
+      </c>
+      <c r="G411">
+        <v>6</v>
+      </c>
+      <c r="H411">
+        <v>90</v>
+      </c>
+      <c r="I411">
+        <v>1</v>
+      </c>
+      <c r="J411">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="412" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A412">
+        <v>21</v>
+      </c>
+      <c r="B412" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C412">
+        <v>21</v>
+      </c>
+      <c r="D412" t="s">
+        <v>51</v>
+      </c>
+      <c r="F412">
+        <v>1</v>
+      </c>
+      <c r="G412">
+        <v>6</v>
+      </c>
+      <c r="H412">
+        <v>90</v>
+      </c>
+      <c r="I412">
+        <v>1</v>
+      </c>
+      <c r="J412">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="413" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A413">
+        <v>21</v>
+      </c>
+      <c r="B413" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C413">
+        <v>21</v>
+      </c>
+      <c r="D413" t="s">
+        <v>51</v>
+      </c>
+      <c r="F413">
+        <v>1</v>
+      </c>
+      <c r="G413">
+        <v>6</v>
+      </c>
+      <c r="H413">
+        <v>90</v>
+      </c>
+      <c r="I413">
+        <v>1</v>
+      </c>
+      <c r="J413">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="414" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A414">
+        <v>21</v>
+      </c>
+      <c r="B414" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C414">
+        <v>21</v>
+      </c>
+      <c r="D414" t="s">
+        <v>51</v>
+      </c>
+      <c r="F414">
+        <v>1</v>
+      </c>
+      <c r="G414">
+        <v>6</v>
+      </c>
+      <c r="H414">
+        <v>90</v>
+      </c>
+      <c r="I414">
+        <v>1</v>
+      </c>
+      <c r="J414">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="415" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A415">
+        <v>21</v>
+      </c>
+      <c r="B415" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C415">
+        <v>21</v>
+      </c>
+      <c r="D415" t="s">
+        <v>51</v>
+      </c>
+      <c r="F415">
+        <v>1</v>
+      </c>
+      <c r="G415">
+        <v>6</v>
+      </c>
+      <c r="H415">
+        <v>90</v>
+      </c>
+      <c r="I415">
+        <v>1</v>
+      </c>
+      <c r="J415">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="416" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A416">
+        <v>21</v>
+      </c>
+      <c r="B416" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C416">
+        <v>21</v>
+      </c>
+      <c r="D416" t="s">
+        <v>51</v>
+      </c>
+      <c r="F416">
+        <v>1</v>
+      </c>
+      <c r="G416">
+        <v>6</v>
+      </c>
+      <c r="H416">
+        <v>3</v>
+      </c>
+      <c r="I416">
+        <v>0</v>
+      </c>
+      <c r="J416">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="417" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A417">
+        <v>21</v>
+      </c>
+      <c r="B417" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C417">
+        <v>21</v>
+      </c>
+      <c r="D417" t="s">
+        <v>51</v>
+      </c>
+      <c r="F417">
+        <v>1</v>
+      </c>
+      <c r="G417">
+        <v>6</v>
+      </c>
+      <c r="H417">
+        <v>33</v>
+      </c>
+      <c r="I417">
+        <v>0</v>
+      </c>
+      <c r="J417">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="418" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A418">
+        <v>21</v>
+      </c>
+      <c r="B418" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C418">
+        <v>21</v>
+      </c>
+      <c r="D418" t="s">
+        <v>51</v>
+      </c>
+      <c r="F418">
+        <v>1</v>
+      </c>
+      <c r="G418">
+        <v>6</v>
+      </c>
+      <c r="H418">
+        <v>5</v>
+      </c>
+      <c r="I418">
+        <v>0</v>
+      </c>
+      <c r="J418">
         <v>1</v>
       </c>
     </row>
@@ -9073,7 +12412,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFDCF622-BAB6-4971-B843-0A581D15DC9C}">
-  <dimension ref="A1:R16"/>
+  <dimension ref="A1:R23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="29.5546875" bestFit="1" customWidth="1"/>
@@ -9133,7 +12472,7 @@
         <v>27</v>
       </c>
       <c r="R1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
@@ -9236,15 +12575,15 @@
         <v>0</v>
       </c>
       <c r="N3">
-        <f t="shared" ref="N3:N16" si="0">SUM(H3:I3)</f>
+        <f t="shared" ref="N3:N22" si="0">SUM(H3:I3)</f>
         <v>1</v>
       </c>
       <c r="O3">
-        <f t="shared" ref="O3:O16" si="1">SUM(J3:K3)</f>
+        <f t="shared" ref="O3:O22" si="1">SUM(J3:K3)</f>
         <v>0</v>
       </c>
       <c r="P3">
-        <f t="shared" ref="P3:P16" si="2">SUM(L3:M3)</f>
+        <f t="shared" ref="P3:P22" si="2">SUM(L3:M3)</f>
         <v>1</v>
       </c>
       <c r="Q3">
@@ -10020,6 +13359,363 @@
       <c r="R16">
         <v>11</v>
       </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" s="1">
+        <v>46054</v>
+      </c>
+      <c r="C17" s="5">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17">
+        <v>11</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17">
+        <v>1</v>
+      </c>
+      <c r="H17">
+        <v>3</v>
+      </c>
+      <c r="I17">
+        <v>3</v>
+      </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17">
+        <v>5</v>
+      </c>
+      <c r="M17">
+        <v>5</v>
+      </c>
+      <c r="N17">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="O17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="P17">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="Q17">
+        <v>18</v>
+      </c>
+      <c r="R17">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" s="1">
+        <v>46060</v>
+      </c>
+      <c r="C18" s="5">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="D18">
+        <v>7</v>
+      </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
+      <c r="F18">
+        <v>3</v>
+      </c>
+      <c r="G18">
+        <v>4</v>
+      </c>
+      <c r="H18">
+        <v>3</v>
+      </c>
+      <c r="I18">
+        <v>4</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <v>5</v>
+      </c>
+      <c r="M18">
+        <v>5</v>
+      </c>
+      <c r="N18">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="O18">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="P18">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="Q18">
+        <v>21</v>
+      </c>
+      <c r="R18">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" s="1">
+        <v>46075</v>
+      </c>
+      <c r="C19" s="5">
+        <v>0.6875</v>
+      </c>
+      <c r="D19">
+        <v>2</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19">
+        <v>5</v>
+      </c>
+      <c r="G19">
+        <v>1</v>
+      </c>
+      <c r="H19">
+        <v>3</v>
+      </c>
+      <c r="I19">
+        <v>4</v>
+      </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
+      <c r="L19">
+        <v>5</v>
+      </c>
+      <c r="M19">
+        <v>6</v>
+      </c>
+      <c r="N19">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="O19">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="P19">
+        <f t="shared" si="2"/>
+        <v>11</v>
+      </c>
+      <c r="Q19">
+        <v>21</v>
+      </c>
+      <c r="R19">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" s="1">
+        <v>46082</v>
+      </c>
+      <c r="C20" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20">
+        <v>15</v>
+      </c>
+      <c r="F20">
+        <v>2</v>
+      </c>
+      <c r="G20">
+        <v>1</v>
+      </c>
+      <c r="H20">
+        <v>4</v>
+      </c>
+      <c r="I20">
+        <v>4</v>
+      </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="L20">
+        <v>5</v>
+      </c>
+      <c r="M20">
+        <v>6</v>
+      </c>
+      <c r="N20">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="O20">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="P20">
+        <f t="shared" si="2"/>
+        <v>11</v>
+      </c>
+      <c r="Q20">
+        <v>24</v>
+      </c>
+      <c r="R20">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" s="1">
+        <v>46089</v>
+      </c>
+      <c r="C21" s="5">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="D21">
+        <v>14</v>
+      </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21">
+        <v>2</v>
+      </c>
+      <c r="G21">
+        <v>1</v>
+      </c>
+      <c r="H21">
+        <v>4</v>
+      </c>
+      <c r="I21">
+        <v>4</v>
+      </c>
+      <c r="J21">
+        <v>0</v>
+      </c>
+      <c r="K21">
+        <v>0</v>
+      </c>
+      <c r="L21">
+        <v>5</v>
+      </c>
+      <c r="M21">
+        <v>7</v>
+      </c>
+      <c r="N21">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="O21">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="P21">
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="Q21">
+        <v>24</v>
+      </c>
+      <c r="R21">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1">
+        <v>46096</v>
+      </c>
+      <c r="C22" s="5">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22">
+        <v>6</v>
+      </c>
+      <c r="F22">
+        <v>2</v>
+      </c>
+      <c r="G22">
+        <v>1</v>
+      </c>
+      <c r="H22">
+        <v>5</v>
+      </c>
+      <c r="I22">
+        <v>4</v>
+      </c>
+      <c r="J22">
+        <v>0</v>
+      </c>
+      <c r="K22">
+        <v>0</v>
+      </c>
+      <c r="L22">
+        <v>5</v>
+      </c>
+      <c r="M22">
+        <v>7</v>
+      </c>
+      <c r="N22">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="O22">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="P22">
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="Q22">
+        <v>27</v>
+      </c>
+      <c r="R22">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="B23" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
dep`loy enviroment for shinyapps.io
</commit_message>
<xml_diff>
--- a/inst/app/data/CAZALEGAS_B_DATA.xlsx
+++ b/inst/app/data/CAZALEGAS_B_DATA.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Equipo\Desktop\MASTER_MUSA\REPOS\FootballTeamTracker\inst\app\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danis\Desktop\MASTER\REPOS\FootballTeamTracker\inst\app\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEA933F1-A961-4B28-BB09-705EB6D56ED8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E295C58-2998-4EDA-8653-C43851319E3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{46C6BD2A-3E4B-49DE-A2D3-07FEC4388880}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{46C6BD2A-3E4B-49DE-A2D3-07FEC4388880}"/>
   </bookViews>
   <sheets>
     <sheet name="Eventos" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="871" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="903" uniqueCount="85">
   <si>
     <t>Jornada</t>
   </si>
@@ -287,6 +287,12 @@
   </si>
   <si>
     <t>Roque Alberto Celaya Rodriguez</t>
+  </si>
+  <si>
+    <t>Gael Isaac Barreras Leyva</t>
+  </si>
+  <si>
+    <t>Matvei Pogadaev</t>
   </si>
 </sst>
 </file>
@@ -669,17 +675,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA997B58-975D-4006-998B-0A230432491C}">
-  <dimension ref="A1:J418"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:J434"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="22.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>28</v>
       </c>
@@ -711,7 +717,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -734,7 +740,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -766,7 +772,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -798,7 +804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -830,7 +836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1</v>
       </c>
@@ -853,7 +859,7 @@
         <v>1</v>
       </c>
       <c r="H6">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="I6">
         <v>1</v>
@@ -862,7 +868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1</v>
       </c>
@@ -885,7 +891,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1</v>
       </c>
@@ -917,7 +923,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1</v>
       </c>
@@ -946,7 +952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1</v>
       </c>
@@ -975,7 +981,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>1</v>
       </c>
@@ -1004,7 +1010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>1</v>
       </c>
@@ -1033,7 +1039,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>1</v>
       </c>
@@ -1062,7 +1068,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>1</v>
       </c>
@@ -1091,7 +1097,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>1</v>
       </c>
@@ -1120,7 +1126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>1</v>
       </c>
@@ -1149,7 +1155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>1</v>
       </c>
@@ -1178,7 +1184,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>1</v>
       </c>
@@ -1207,7 +1213,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>1</v>
       </c>
@@ -1236,7 +1242,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>1</v>
       </c>
@@ -1265,7 +1271,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>1</v>
       </c>
@@ -1288,7 +1294,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>1</v>
       </c>
@@ -1311,7 +1317,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>1</v>
       </c>
@@ -1334,7 +1340,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2</v>
       </c>
@@ -1357,7 +1363,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2</v>
       </c>
@@ -1380,7 +1386,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2</v>
       </c>
@@ -1403,7 +1409,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2</v>
       </c>
@@ -1435,7 +1441,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2</v>
       </c>
@@ -1467,7 +1473,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>2</v>
       </c>
@@ -1496,7 +1502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>2</v>
       </c>
@@ -1525,7 +1531,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2</v>
       </c>
@@ -1554,7 +1560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>2</v>
       </c>
@@ -1583,7 +1589,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>2</v>
       </c>
@@ -1612,7 +1618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>2</v>
       </c>
@@ -1641,7 +1647,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>2</v>
       </c>
@@ -1670,7 +1676,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>2</v>
       </c>
@@ -1699,7 +1705,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>2</v>
       </c>
@@ -1728,7 +1734,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>2</v>
       </c>
@@ -1757,7 +1763,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>2</v>
       </c>
@@ -1786,7 +1792,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>2</v>
       </c>
@@ -1815,7 +1821,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>2</v>
       </c>
@@ -1844,7 +1850,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>2</v>
       </c>
@@ -1873,7 +1879,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>2</v>
       </c>
@@ -1902,7 +1908,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>3</v>
       </c>
@@ -1934,7 +1940,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>3</v>
       </c>
@@ -1957,7 +1963,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>3</v>
       </c>
@@ -1980,7 +1986,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>3</v>
       </c>
@@ -2003,7 +2009,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>3</v>
       </c>
@@ -2026,7 +2032,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>3</v>
       </c>
@@ -2049,7 +2055,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>3</v>
       </c>
@@ -2072,7 +2078,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>3</v>
       </c>
@@ -2095,7 +2101,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>3</v>
       </c>
@@ -2124,7 +2130,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>3</v>
       </c>
@@ -2153,7 +2159,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>3</v>
       </c>
@@ -2182,7 +2188,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>3</v>
       </c>
@@ -2211,7 +2217,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>3</v>
       </c>
@@ -2240,7 +2246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>3</v>
       </c>
@@ -2269,7 +2275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>3</v>
       </c>
@@ -2298,7 +2304,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>3</v>
       </c>
@@ -2327,7 +2333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>3</v>
       </c>
@@ -2356,7 +2362,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>3</v>
       </c>
@@ -2385,7 +2391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>3</v>
       </c>
@@ -2414,7 +2420,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>3</v>
       </c>
@@ -2443,7 +2449,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>3</v>
       </c>
@@ -2472,7 +2478,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>3</v>
       </c>
@@ -2501,7 +2507,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>3</v>
       </c>
@@ -2530,7 +2536,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>3</v>
       </c>
@@ -2559,7 +2565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>4</v>
       </c>
@@ -2582,7 +2588,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>4</v>
       </c>
@@ -2605,7 +2611,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>4</v>
       </c>
@@ -2628,7 +2634,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>4</v>
       </c>
@@ -2651,7 +2657,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>4</v>
       </c>
@@ -2683,7 +2689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>4</v>
       </c>
@@ -2706,7 +2712,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>4</v>
       </c>
@@ -2729,7 +2735,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>4</v>
       </c>
@@ -2761,7 +2767,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>4</v>
       </c>
@@ -2793,7 +2799,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>4</v>
       </c>
@@ -2825,7 +2831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>4</v>
       </c>
@@ -2857,7 +2863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>4</v>
       </c>
@@ -2889,7 +2895,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>4</v>
       </c>
@@ -2918,7 +2924,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>4</v>
       </c>
@@ -2947,7 +2953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>4</v>
       </c>
@@ -2976,7 +2982,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>4</v>
       </c>
@@ -3005,7 +3011,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>4</v>
       </c>
@@ -3034,7 +3040,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>4</v>
       </c>
@@ -3063,7 +3069,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>4</v>
       </c>
@@ -3092,7 +3098,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>4</v>
       </c>
@@ -3121,7 +3127,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>4</v>
       </c>
@@ -3150,7 +3156,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>5</v>
       </c>
@@ -3173,7 +3179,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>5</v>
       </c>
@@ -3196,7 +3202,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>5</v>
       </c>
@@ -3219,7 +3225,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>5</v>
       </c>
@@ -3242,7 +3248,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>5</v>
       </c>
@@ -3274,7 +3280,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>5</v>
       </c>
@@ -3306,7 +3312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>5</v>
       </c>
@@ -3338,7 +3344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>5</v>
       </c>
@@ -3370,7 +3376,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>5</v>
       </c>
@@ -3402,7 +3408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>5</v>
       </c>
@@ -3434,7 +3440,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>5</v>
       </c>
@@ -3463,7 +3469,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>5</v>
       </c>
@@ -3492,7 +3498,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>5</v>
       </c>
@@ -3521,7 +3527,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>5</v>
       </c>
@@ -3550,7 +3556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>5</v>
       </c>
@@ -3579,7 +3585,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>5</v>
       </c>
@@ -3608,7 +3614,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>5</v>
       </c>
@@ -3637,7 +3643,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>5</v>
       </c>
@@ -3666,7 +3672,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>6</v>
       </c>
@@ -3689,7 +3695,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>6</v>
       </c>
@@ -3712,7 +3718,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>6</v>
       </c>
@@ -3735,7 +3741,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>6</v>
       </c>
@@ -3758,7 +3764,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>6</v>
       </c>
@@ -3781,7 +3787,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>6</v>
       </c>
@@ -3804,7 +3810,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>6</v>
       </c>
@@ -3827,7 +3833,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>6</v>
       </c>
@@ -3859,7 +3865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>6</v>
       </c>
@@ -3888,7 +3894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>6</v>
       </c>
@@ -3917,7 +3923,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>6</v>
       </c>
@@ -3946,7 +3952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>6</v>
       </c>
@@ -3975,7 +3981,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>6</v>
       </c>
@@ -4004,7 +4010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>6</v>
       </c>
@@ -4033,7 +4039,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>6</v>
       </c>
@@ -4062,7 +4068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>6</v>
       </c>
@@ -4091,7 +4097,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>6</v>
       </c>
@@ -4120,7 +4126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>6</v>
       </c>
@@ -4149,7 +4155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>6</v>
       </c>
@@ -4178,7 +4184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>6</v>
       </c>
@@ -4207,7 +4213,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>6</v>
       </c>
@@ -4236,7 +4242,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>7</v>
       </c>
@@ -4259,7 +4265,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>7</v>
       </c>
@@ -4282,7 +4288,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>7</v>
       </c>
@@ -4305,7 +4311,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>7</v>
       </c>
@@ -4328,7 +4334,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>7</v>
       </c>
@@ -4360,7 +4366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>7</v>
       </c>
@@ -4392,7 +4398,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>7</v>
       </c>
@@ -4424,7 +4430,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>7</v>
       </c>
@@ -4456,7 +4462,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>7</v>
       </c>
@@ -4488,7 +4494,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>7</v>
       </c>
@@ -4517,7 +4523,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>7</v>
       </c>
@@ -4546,7 +4552,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>7</v>
       </c>
@@ -4575,7 +4581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>7</v>
       </c>
@@ -4604,7 +4610,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>7</v>
       </c>
@@ -4633,7 +4639,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>7</v>
       </c>
@@ -4662,7 +4668,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>7</v>
       </c>
@@ -4691,7 +4697,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>7</v>
       </c>
@@ -4720,7 +4726,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>7</v>
       </c>
@@ -4749,7 +4755,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>7</v>
       </c>
@@ -4778,7 +4784,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>7</v>
       </c>
@@ -4807,7 +4813,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>8</v>
       </c>
@@ -4830,7 +4836,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="149" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>8</v>
       </c>
@@ -4853,7 +4859,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>8</v>
       </c>
@@ -4885,7 +4891,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>8</v>
       </c>
@@ -4917,7 +4923,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>8</v>
       </c>
@@ -4949,7 +4955,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>8</v>
       </c>
@@ -4981,7 +4987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>8</v>
       </c>
@@ -5013,7 +5019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>8</v>
       </c>
@@ -5042,7 +5048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A156">
         <v>8</v>
       </c>
@@ -5071,7 +5077,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A157">
         <v>8</v>
       </c>
@@ -5100,7 +5106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A158">
         <v>8</v>
       </c>
@@ -5129,7 +5135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>8</v>
       </c>
@@ -5158,7 +5164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>8</v>
       </c>
@@ -5187,7 +5193,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="161" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>8</v>
       </c>
@@ -5216,7 +5222,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A162">
         <v>8</v>
       </c>
@@ -5245,7 +5251,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="163" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A163">
         <v>8</v>
       </c>
@@ -5274,7 +5280,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="164" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>9</v>
       </c>
@@ -5297,7 +5303,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="165" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>9</v>
       </c>
@@ -5320,7 +5326,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="166" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>9</v>
       </c>
@@ -5343,7 +5349,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="167" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A167">
         <v>9</v>
       </c>
@@ -5366,7 +5372,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="168" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A168">
         <v>9</v>
       </c>
@@ -5389,7 +5395,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="169" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A169">
         <v>9</v>
       </c>
@@ -5412,7 +5418,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="170" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>9</v>
       </c>
@@ -5444,7 +5450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A171">
         <v>9</v>
       </c>
@@ -5476,7 +5482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A172">
         <v>9</v>
       </c>
@@ -5508,7 +5514,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="173" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A173">
         <v>9</v>
       </c>
@@ -5537,7 +5543,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A174">
         <v>9</v>
       </c>
@@ -5566,7 +5572,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="175" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A175">
         <v>9</v>
       </c>
@@ -5595,7 +5601,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A176">
         <v>9</v>
       </c>
@@ -5624,7 +5630,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A177">
         <v>9</v>
       </c>
@@ -5653,7 +5659,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A178">
         <v>9</v>
       </c>
@@ -5682,7 +5688,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="179" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A179">
         <v>9</v>
       </c>
@@ -5711,7 +5717,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="180" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>9</v>
       </c>
@@ -5740,7 +5746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>9</v>
       </c>
@@ -5769,7 +5775,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="182" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A182">
         <v>9</v>
       </c>
@@ -5798,7 +5804,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="183" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A183">
         <v>9</v>
       </c>
@@ -5827,7 +5833,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="184" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A184">
         <v>9</v>
       </c>
@@ -5856,7 +5862,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="185" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A185">
         <v>9</v>
       </c>
@@ -5885,7 +5891,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A186">
         <v>9</v>
       </c>
@@ -5914,7 +5920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A187">
         <v>10</v>
       </c>
@@ -5937,7 +5943,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="188" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A188">
         <v>10</v>
       </c>
@@ -5960,7 +5966,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="189" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A189">
         <v>10</v>
       </c>
@@ -5983,7 +5989,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A190">
         <v>10</v>
       </c>
@@ -6006,7 +6012,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="191" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A191">
         <v>10</v>
       </c>
@@ -6038,7 +6044,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A192">
         <v>10</v>
       </c>
@@ -6070,7 +6076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A193">
         <v>10</v>
       </c>
@@ -6099,7 +6105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A194">
         <v>10</v>
       </c>
@@ -6128,7 +6134,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A195">
         <v>10</v>
       </c>
@@ -6157,7 +6163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A196">
         <v>10</v>
       </c>
@@ -6186,7 +6192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A197">
         <v>10</v>
       </c>
@@ -6215,7 +6221,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="198" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A198">
         <v>10</v>
       </c>
@@ -6244,7 +6250,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="199" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A199">
         <v>10</v>
       </c>
@@ -6273,7 +6279,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="200" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A200">
         <v>10</v>
       </c>
@@ -6302,7 +6308,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A201">
         <v>10</v>
       </c>
@@ -6331,7 +6337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A202">
         <v>10</v>
       </c>
@@ -6360,7 +6366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A203">
         <v>10</v>
       </c>
@@ -6389,7 +6395,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="204" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A204">
         <v>10</v>
       </c>
@@ -6418,7 +6424,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A205">
         <v>10</v>
       </c>
@@ -6447,7 +6453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A206">
         <v>10</v>
       </c>
@@ -6476,7 +6482,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="207" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A207">
         <v>11</v>
       </c>
@@ -6499,7 +6505,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="208" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A208">
         <v>11</v>
       </c>
@@ -6522,7 +6528,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="209" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A209">
         <v>11</v>
       </c>
@@ -6545,7 +6551,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="210" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A210">
         <v>11</v>
       </c>
@@ -6568,7 +6574,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="211" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A211">
         <v>11</v>
       </c>
@@ -6591,7 +6597,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="212" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A212">
         <v>11</v>
       </c>
@@ -6614,7 +6620,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="213" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A213">
         <v>11</v>
       </c>
@@ -6637,7 +6643,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="214" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A214">
         <v>11</v>
       </c>
@@ -6660,7 +6666,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="215" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A215">
         <v>11</v>
       </c>
@@ -6692,7 +6698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A216">
         <v>11</v>
       </c>
@@ -6724,7 +6730,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="217" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A217">
         <v>11</v>
       </c>
@@ -6756,7 +6762,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A218">
         <v>11</v>
       </c>
@@ -6788,7 +6794,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="219" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A219">
         <v>11</v>
       </c>
@@ -6820,7 +6826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A220">
         <v>11</v>
       </c>
@@ -6849,7 +6855,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A221">
         <v>11</v>
       </c>
@@ -6878,7 +6884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A222">
         <v>11</v>
       </c>
@@ -6907,7 +6913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A223">
         <v>11</v>
       </c>
@@ -6936,7 +6942,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A224">
         <v>11</v>
       </c>
@@ -6965,7 +6971,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="225" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A225">
         <v>11</v>
       </c>
@@ -6994,7 +7000,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="226" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A226">
         <v>11</v>
       </c>
@@ -7023,7 +7029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A227">
         <v>11</v>
       </c>
@@ -7052,7 +7058,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A228">
         <v>11</v>
       </c>
@@ -7081,7 +7087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A229">
         <v>11</v>
       </c>
@@ -7110,7 +7116,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="230" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A230">
         <v>11</v>
       </c>
@@ -7139,7 +7145,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="231" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A231">
         <v>11</v>
       </c>
@@ -7168,7 +7174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="232" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A232">
         <v>11</v>
       </c>
@@ -7197,7 +7203,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="233" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A233">
         <v>12</v>
       </c>
@@ -7220,7 +7226,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="234" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A234">
         <v>12</v>
       </c>
@@ -7243,7 +7249,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="235" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A235">
         <v>12</v>
       </c>
@@ -7266,7 +7272,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="236" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A236">
         <v>12</v>
       </c>
@@ -7298,7 +7304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="237" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A237">
         <v>12</v>
       </c>
@@ -7330,7 +7336,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="238" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A238">
         <v>12</v>
       </c>
@@ -7362,7 +7368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="239" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A239">
         <v>12</v>
       </c>
@@ -7394,7 +7400,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="240" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A240">
         <v>12</v>
       </c>
@@ -7420,7 +7426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="241" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A241">
         <v>12</v>
       </c>
@@ -7446,7 +7452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="242" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A242">
         <v>12</v>
       </c>
@@ -7472,7 +7478,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="243" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A243">
         <v>12</v>
       </c>
@@ -7498,7 +7504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="244" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A244">
         <v>12</v>
       </c>
@@ -7524,7 +7530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="245" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A245">
         <v>12</v>
       </c>
@@ -7550,7 +7556,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="246" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A246">
         <v>12</v>
       </c>
@@ -7576,7 +7582,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="247" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A247">
         <v>12</v>
       </c>
@@ -7602,7 +7608,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="248" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A248">
         <v>12</v>
       </c>
@@ -7628,7 +7634,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="249" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A249">
         <v>12</v>
       </c>
@@ -7654,7 +7660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="250" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A250">
         <v>13</v>
       </c>
@@ -7677,7 +7683,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="251" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A251">
         <v>13</v>
       </c>
@@ -7700,7 +7706,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="252" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A252">
         <v>13</v>
       </c>
@@ -7723,7 +7729,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="253" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A253">
         <v>13</v>
       </c>
@@ -7746,7 +7752,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="254" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A254">
         <v>13</v>
       </c>
@@ -7778,7 +7784,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="255" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A255">
         <v>13</v>
       </c>
@@ -7807,7 +7813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="256" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A256">
         <v>13</v>
       </c>
@@ -7836,7 +7842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="257" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A257">
         <v>13</v>
       </c>
@@ -7865,7 +7871,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="258" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A258">
         <v>13</v>
       </c>
@@ -7894,7 +7900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="259" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A259">
         <v>13</v>
       </c>
@@ -7923,7 +7929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="260" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A260">
         <v>13</v>
       </c>
@@ -7952,7 +7958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="261" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A261">
         <v>13</v>
       </c>
@@ -7981,7 +7987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="262" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A262">
         <v>13</v>
       </c>
@@ -8010,7 +8016,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="263" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A263">
         <v>13</v>
       </c>
@@ -8039,7 +8045,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="264" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A264">
         <v>13</v>
       </c>
@@ -8068,7 +8074,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="265" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A265">
         <v>13</v>
       </c>
@@ -8097,7 +8103,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="266" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A266">
         <v>13</v>
       </c>
@@ -8126,7 +8132,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="267" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A267">
         <v>13</v>
       </c>
@@ -8155,7 +8161,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="268" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A268">
         <v>13</v>
       </c>
@@ -8184,7 +8190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="269" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A269">
         <v>14</v>
       </c>
@@ -8207,7 +8213,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="270" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A270">
         <v>14</v>
       </c>
@@ -8230,7 +8236,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="271" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A271">
         <v>14</v>
       </c>
@@ -8253,7 +8259,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="272" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A272">
         <v>14</v>
       </c>
@@ -8285,7 +8291,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="273" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A273">
         <v>14</v>
       </c>
@@ -8314,7 +8320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="274" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A274">
         <v>14</v>
       </c>
@@ -8343,7 +8349,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="275" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A275">
         <v>14</v>
       </c>
@@ -8372,7 +8378,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="276" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A276">
         <v>14</v>
       </c>
@@ -8401,7 +8407,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="277" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A277">
         <v>14</v>
       </c>
@@ -8430,7 +8436,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="278" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A278">
         <v>14</v>
       </c>
@@ -8459,7 +8465,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="279" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A279">
         <v>14</v>
       </c>
@@ -8488,7 +8494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="280" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A280">
         <v>14</v>
       </c>
@@ -8517,7 +8523,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="281" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A281">
         <v>14</v>
       </c>
@@ -8546,7 +8552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="282" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A282">
         <v>14</v>
       </c>
@@ -8575,7 +8581,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="283" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A283">
         <v>14</v>
       </c>
@@ -8604,7 +8610,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="284" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A284">
         <v>14</v>
       </c>
@@ -8633,7 +8639,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="285" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A285">
         <v>14</v>
       </c>
@@ -8662,7 +8668,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="286" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A286">
         <v>15</v>
       </c>
@@ -8685,7 +8691,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="287" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A287">
         <v>15</v>
       </c>
@@ -8717,7 +8723,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="288" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A288">
         <v>15</v>
       </c>
@@ -8749,7 +8755,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="289" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A289">
         <v>15</v>
       </c>
@@ -8778,7 +8784,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="290" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A290">
         <v>15</v>
       </c>
@@ -8807,7 +8813,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="291" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A291">
         <v>15</v>
       </c>
@@ -8836,7 +8842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="292" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A292">
         <v>15</v>
       </c>
@@ -8865,7 +8871,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="293" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A293">
         <v>15</v>
       </c>
@@ -8894,7 +8900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="294" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A294">
         <v>15</v>
       </c>
@@ -8923,7 +8929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="295" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A295">
         <v>15</v>
       </c>
@@ -8952,7 +8958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="296" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A296">
         <v>15</v>
       </c>
@@ -8981,7 +8987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="297" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A297">
         <v>15</v>
       </c>
@@ -9010,7 +9016,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="298" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A298">
         <v>15</v>
       </c>
@@ -9039,7 +9045,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="299" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A299">
         <v>15</v>
       </c>
@@ -9068,7 +9074,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="300" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A300">
         <v>16</v>
       </c>
@@ -9091,7 +9097,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="301" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A301">
         <v>16</v>
       </c>
@@ -9114,7 +9120,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="302" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A302">
         <v>16</v>
       </c>
@@ -9146,7 +9152,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="303" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A303">
         <v>16</v>
       </c>
@@ -9178,7 +9184,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="304" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A304">
         <v>16</v>
       </c>
@@ -9207,7 +9213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="305" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A305">
         <v>16</v>
       </c>
@@ -9236,7 +9242,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="306" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A306">
         <v>16</v>
       </c>
@@ -9265,7 +9271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="307" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A307">
         <v>16</v>
       </c>
@@ -9294,7 +9300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="308" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A308">
         <v>16</v>
       </c>
@@ -9323,7 +9329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="309" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A309">
         <v>16</v>
       </c>
@@ -9352,7 +9358,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="310" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A310">
         <v>16</v>
       </c>
@@ -9381,7 +9387,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="311" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A311">
         <v>16</v>
       </c>
@@ -9410,7 +9416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="312" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A312">
         <v>16</v>
       </c>
@@ -9439,7 +9445,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="313" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A313">
         <v>16</v>
       </c>
@@ -9468,7 +9474,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="314" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A314">
         <v>16</v>
       </c>
@@ -9497,7 +9503,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="315" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A315">
         <v>16</v>
       </c>
@@ -9526,7 +9532,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="316" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A316">
         <v>16</v>
       </c>
@@ -9555,7 +9561,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="317" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A317">
         <v>16</v>
       </c>
@@ -9584,7 +9590,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="318" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A318">
         <v>17</v>
       </c>
@@ -9607,7 +9613,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="319" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A319">
         <v>17</v>
       </c>
@@ -9630,7 +9636,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="320" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A320">
         <v>17</v>
       </c>
@@ -9653,7 +9659,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="321" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A321">
         <v>17</v>
       </c>
@@ -9676,7 +9682,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="322" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A322">
         <v>17</v>
       </c>
@@ -9708,7 +9714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="323" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A323">
         <v>17</v>
       </c>
@@ -9740,7 +9746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="324" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A324">
         <v>17</v>
       </c>
@@ -9772,7 +9778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="325" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A325">
         <v>17</v>
       </c>
@@ -9804,7 +9810,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="326" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A326">
         <v>17</v>
       </c>
@@ -9836,7 +9842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="327" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A327">
         <v>17</v>
       </c>
@@ -9868,7 +9874,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="328" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A328">
         <v>17</v>
       </c>
@@ -9897,7 +9903,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="329" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A329">
         <v>17</v>
       </c>
@@ -9926,7 +9932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="330" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A330">
         <v>17</v>
       </c>
@@ -9955,7 +9961,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="331" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A331">
         <v>17</v>
       </c>
@@ -9984,7 +9990,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="332" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A332">
         <v>17</v>
       </c>
@@ -10013,7 +10019,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="333" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A333">
         <v>17</v>
       </c>
@@ -10042,7 +10048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="334" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A334">
         <v>17</v>
       </c>
@@ -10071,7 +10077,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="335" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A335">
         <v>17</v>
       </c>
@@ -10100,7 +10106,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="336" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A336">
         <v>17</v>
       </c>
@@ -10129,7 +10135,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="337" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A337">
         <v>18</v>
       </c>
@@ -10152,7 +10158,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="338" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A338">
         <v>18</v>
       </c>
@@ -10175,7 +10181,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="339" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A339">
         <v>18</v>
       </c>
@@ -10198,7 +10204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="340" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A340">
         <v>18</v>
       </c>
@@ -10221,7 +10227,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="341" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A341">
         <v>18</v>
       </c>
@@ -10244,7 +10250,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="342" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="342" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A342">
         <v>18</v>
       </c>
@@ -10267,7 +10273,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="343" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A343">
         <v>18</v>
       </c>
@@ -10290,7 +10296,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="344" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A344">
         <v>18</v>
       </c>
@@ -10322,7 +10328,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="345" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="345" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A345">
         <v>18</v>
       </c>
@@ -10354,7 +10360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="346" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A346">
         <v>18</v>
       </c>
@@ -10386,7 +10392,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="347" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A347">
         <v>18</v>
       </c>
@@ -10415,7 +10421,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="348" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A348">
         <v>18</v>
       </c>
@@ -10444,7 +10450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="349" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A349">
         <v>18</v>
       </c>
@@ -10473,7 +10479,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="350" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A350">
         <v>18</v>
       </c>
@@ -10502,7 +10508,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="351" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A351">
         <v>18</v>
       </c>
@@ -10531,7 +10537,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="352" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A352">
         <v>18</v>
       </c>
@@ -10560,7 +10566,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="353" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A353">
         <v>18</v>
       </c>
@@ -10589,7 +10595,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="354" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="354" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A354">
         <v>18</v>
       </c>
@@ -10618,7 +10624,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="355" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="355" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A355">
         <v>18</v>
       </c>
@@ -10647,7 +10653,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="356" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A356">
         <v>18</v>
       </c>
@@ -10676,7 +10682,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="357" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="357" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A357">
         <v>19</v>
       </c>
@@ -10699,7 +10705,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="358" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A358">
         <v>19</v>
       </c>
@@ -10722,7 +10728,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="359" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A359">
         <v>19</v>
       </c>
@@ -10745,7 +10751,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="360" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A360">
         <v>19</v>
       </c>
@@ -10768,7 +10774,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="361" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="361" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A361">
         <v>19</v>
       </c>
@@ -10791,7 +10797,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="362" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="362" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A362">
         <v>19</v>
       </c>
@@ -10823,7 +10829,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="363" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="363" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A363">
         <v>19</v>
       </c>
@@ -10855,7 +10861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="364" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="364" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A364">
         <v>19</v>
       </c>
@@ -10887,7 +10893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="365" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A365">
         <v>19</v>
       </c>
@@ -10916,7 +10922,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="366" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="366" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A366">
         <v>19</v>
       </c>
@@ -10945,7 +10951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="367" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="367" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A367">
         <v>19</v>
       </c>
@@ -10974,7 +10980,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="368" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="368" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A368">
         <v>19</v>
       </c>
@@ -11003,7 +11009,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="369" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="369" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A369">
         <v>19</v>
       </c>
@@ -11032,7 +11038,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="370" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="370" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A370">
         <v>19</v>
       </c>
@@ -11061,7 +11067,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="371" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="371" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A371">
         <v>19</v>
       </c>
@@ -11090,7 +11096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="372" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="372" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A372">
         <v>19</v>
       </c>
@@ -11119,7 +11125,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="373" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="373" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A373">
         <v>19</v>
       </c>
@@ -11148,7 +11154,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="374" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="374" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A374">
         <v>19</v>
       </c>
@@ -11177,7 +11183,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="375" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="375" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A375">
         <v>20</v>
       </c>
@@ -11200,7 +11206,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="376" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="376" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A376">
         <v>20</v>
       </c>
@@ -11223,7 +11229,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="377" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A377">
         <v>20</v>
       </c>
@@ -11246,7 +11252,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="378" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="378" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A378">
         <v>20</v>
       </c>
@@ -11269,7 +11275,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="379" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="379" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A379">
         <v>20</v>
       </c>
@@ -11292,7 +11298,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="380" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="380" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A380">
         <v>20</v>
       </c>
@@ -11315,7 +11321,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="381" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="381" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A381">
         <v>20</v>
       </c>
@@ -11347,7 +11353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="382" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="382" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A382">
         <v>20</v>
       </c>
@@ -11379,7 +11385,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="383" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="383" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A383">
         <v>20</v>
       </c>
@@ -11411,7 +11417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="384" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="384" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A384">
         <v>20</v>
       </c>
@@ -11443,7 +11449,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="385" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="385" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A385">
         <v>20</v>
       </c>
@@ -11472,7 +11478,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="386" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="386" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A386">
         <v>20</v>
       </c>
@@ -11501,7 +11507,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="387" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A387">
         <v>20</v>
       </c>
@@ -11530,7 +11536,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="388" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="388" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A388">
         <v>20</v>
       </c>
@@ -11559,7 +11565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="389" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="389" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A389">
         <v>20</v>
       </c>
@@ -11588,7 +11594,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="390" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="390" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A390">
         <v>20</v>
       </c>
@@ -11617,7 +11623,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="391" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="391" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A391">
         <v>20</v>
       </c>
@@ -11646,7 +11652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="392" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="392" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A392">
         <v>20</v>
       </c>
@@ -11675,7 +11681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="393" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="393" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A393">
         <v>20</v>
       </c>
@@ -11704,7 +11710,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="394" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="394" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A394">
         <v>20</v>
       </c>
@@ -11733,7 +11739,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="395" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="395" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A395">
         <v>20</v>
       </c>
@@ -11762,7 +11768,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="396" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="396" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A396">
         <v>21</v>
       </c>
@@ -11785,7 +11791,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="397" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="397" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A397">
         <v>21</v>
       </c>
@@ -11808,7 +11814,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="398" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="398" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A398">
         <v>21</v>
       </c>
@@ -11831,7 +11837,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="399" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="399" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A399">
         <v>21</v>
       </c>
@@ -11854,7 +11860,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="400" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="400" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A400">
         <v>21</v>
       </c>
@@ -11877,7 +11883,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="401" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="401" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A401">
         <v>21</v>
       </c>
@@ -11900,7 +11906,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="402" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="402" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A402">
         <v>21</v>
       </c>
@@ -11923,7 +11929,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="403" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="403" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A403">
         <v>21</v>
       </c>
@@ -11955,7 +11961,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="404" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="404" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A404">
         <v>21</v>
       </c>
@@ -11987,7 +11993,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="405" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="405" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A405">
         <v>21</v>
       </c>
@@ -12019,7 +12025,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="406" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="406" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A406">
         <v>21</v>
       </c>
@@ -12051,7 +12057,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="407" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="407" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A407">
         <v>21</v>
       </c>
@@ -12083,7 +12089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="408" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="408" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A408">
         <v>21</v>
       </c>
@@ -12115,7 +12121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="409" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="409" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A409">
         <v>21</v>
       </c>
@@ -12144,7 +12150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="410" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="410" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A410">
         <v>21</v>
       </c>
@@ -12173,7 +12179,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="411" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="411" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A411">
         <v>21</v>
       </c>
@@ -12202,7 +12208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="412" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="412" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A412">
         <v>21</v>
       </c>
@@ -12231,7 +12237,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="413" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="413" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A413">
         <v>21</v>
       </c>
@@ -12260,7 +12266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="414" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="414" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A414">
         <v>21</v>
       </c>
@@ -12289,7 +12295,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="415" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="415" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A415">
         <v>21</v>
       </c>
@@ -12318,7 +12324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="416" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="416" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A416">
         <v>21</v>
       </c>
@@ -12347,7 +12353,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="417" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="417" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A417">
         <v>21</v>
       </c>
@@ -12376,7 +12382,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="418" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="418" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A418">
         <v>21</v>
       </c>
@@ -12403,6 +12409,455 @@
       </c>
       <c r="J418">
         <v>1</v>
+      </c>
+    </row>
+    <row r="419" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A419">
+        <v>22</v>
+      </c>
+      <c r="B419" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C419">
+        <v>22</v>
+      </c>
+      <c r="D419" t="s">
+        <v>26</v>
+      </c>
+      <c r="E419">
+        <v>39</v>
+      </c>
+      <c r="F419">
+        <v>10</v>
+      </c>
+      <c r="G419">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="420" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A420">
+        <v>22</v>
+      </c>
+      <c r="B420" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C420">
+        <v>22</v>
+      </c>
+      <c r="D420" t="s">
+        <v>49</v>
+      </c>
+      <c r="E420">
+        <v>45</v>
+      </c>
+      <c r="F420">
+        <v>10</v>
+      </c>
+      <c r="G420">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="421" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A421">
+        <v>22</v>
+      </c>
+      <c r="B421" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C421">
+        <v>22</v>
+      </c>
+      <c r="D421" t="s">
+        <v>49</v>
+      </c>
+      <c r="E421">
+        <v>55</v>
+      </c>
+      <c r="F421">
+        <v>10</v>
+      </c>
+      <c r="G421">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="422" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A422">
+        <v>22</v>
+      </c>
+      <c r="B422" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C422">
+        <v>22</v>
+      </c>
+      <c r="D422" t="s">
+        <v>49</v>
+      </c>
+      <c r="E422">
+        <v>88</v>
+      </c>
+      <c r="F422">
+        <v>10</v>
+      </c>
+      <c r="G422">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="423" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A423">
+        <v>22</v>
+      </c>
+      <c r="B423" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C423">
+        <v>22</v>
+      </c>
+      <c r="D423" t="s">
+        <v>26</v>
+      </c>
+      <c r="E423">
+        <v>22</v>
+      </c>
+      <c r="F423">
+        <v>10</v>
+      </c>
+      <c r="G423">
+        <v>1</v>
+      </c>
+      <c r="H423">
+        <v>78</v>
+      </c>
+      <c r="I423">
+        <v>1</v>
+      </c>
+      <c r="J423">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="424" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A424">
+        <v>22</v>
+      </c>
+      <c r="B424" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C424">
+        <v>22</v>
+      </c>
+      <c r="D424" t="s">
+        <v>71</v>
+      </c>
+      <c r="E424">
+        <v>87</v>
+      </c>
+      <c r="F424">
+        <v>10</v>
+      </c>
+      <c r="G424">
+        <v>1</v>
+      </c>
+      <c r="H424">
+        <v>12</v>
+      </c>
+      <c r="I424">
+        <v>0</v>
+      </c>
+      <c r="J424">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="425" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A425">
+        <v>22</v>
+      </c>
+      <c r="B425" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C425">
+        <v>22</v>
+      </c>
+      <c r="D425" t="s">
+        <v>49</v>
+      </c>
+      <c r="E425">
+        <v>48</v>
+      </c>
+      <c r="F425">
+        <v>10</v>
+      </c>
+      <c r="G425">
+        <v>1</v>
+      </c>
+      <c r="H425">
+        <v>26</v>
+      </c>
+      <c r="I425">
+        <v>0</v>
+      </c>
+      <c r="J425">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="426" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A426">
+        <v>22</v>
+      </c>
+      <c r="B426" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C426">
+        <v>22</v>
+      </c>
+      <c r="D426" t="s">
+        <v>51</v>
+      </c>
+      <c r="F426">
+        <v>10</v>
+      </c>
+      <c r="G426">
+        <v>1</v>
+      </c>
+      <c r="H426">
+        <v>90</v>
+      </c>
+      <c r="I426">
+        <v>1</v>
+      </c>
+      <c r="J426">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="427" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A427">
+        <v>22</v>
+      </c>
+      <c r="B427" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C427">
+        <v>22</v>
+      </c>
+      <c r="D427" t="s">
+        <v>51</v>
+      </c>
+      <c r="F427">
+        <v>10</v>
+      </c>
+      <c r="G427">
+        <v>1</v>
+      </c>
+      <c r="H427">
+        <v>90</v>
+      </c>
+      <c r="I427">
+        <v>1</v>
+      </c>
+      <c r="J427">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="428" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A428">
+        <v>22</v>
+      </c>
+      <c r="B428" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C428">
+        <v>22</v>
+      </c>
+      <c r="D428" t="s">
+        <v>51</v>
+      </c>
+      <c r="F428">
+        <v>10</v>
+      </c>
+      <c r="G428">
+        <v>1</v>
+      </c>
+      <c r="H428">
+        <v>90</v>
+      </c>
+      <c r="I428">
+        <v>1</v>
+      </c>
+      <c r="J428">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="429" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A429">
+        <v>22</v>
+      </c>
+      <c r="B429" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C429">
+        <v>22</v>
+      </c>
+      <c r="D429" t="s">
+        <v>51</v>
+      </c>
+      <c r="F429">
+        <v>10</v>
+      </c>
+      <c r="G429">
+        <v>1</v>
+      </c>
+      <c r="H429">
+        <v>90</v>
+      </c>
+      <c r="I429">
+        <v>1</v>
+      </c>
+      <c r="J429">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="430" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A430">
+        <v>22</v>
+      </c>
+      <c r="B430" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C430">
+        <v>22</v>
+      </c>
+      <c r="D430" t="s">
+        <v>51</v>
+      </c>
+      <c r="F430">
+        <v>10</v>
+      </c>
+      <c r="G430">
+        <v>1</v>
+      </c>
+      <c r="H430">
+        <v>90</v>
+      </c>
+      <c r="I430">
+        <v>1</v>
+      </c>
+      <c r="J430">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="431" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A431">
+        <v>22</v>
+      </c>
+      <c r="B431" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C431">
+        <v>22</v>
+      </c>
+      <c r="D431" t="s">
+        <v>51</v>
+      </c>
+      <c r="F431">
+        <v>10</v>
+      </c>
+      <c r="G431">
+        <v>1</v>
+      </c>
+      <c r="H431">
+        <v>64</v>
+      </c>
+      <c r="I431">
+        <v>1</v>
+      </c>
+      <c r="J431">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="432" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A432">
+        <v>22</v>
+      </c>
+      <c r="B432" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C432">
+        <v>22</v>
+      </c>
+      <c r="D432" t="s">
+        <v>51</v>
+      </c>
+      <c r="F432">
+        <v>10</v>
+      </c>
+      <c r="G432">
+        <v>1</v>
+      </c>
+      <c r="H432">
+        <v>90</v>
+      </c>
+      <c r="I432">
+        <v>1</v>
+      </c>
+      <c r="J432">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="433" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A433">
+        <v>22</v>
+      </c>
+      <c r="B433" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C433">
+        <v>22</v>
+      </c>
+      <c r="D433" t="s">
+        <v>51</v>
+      </c>
+      <c r="F433">
+        <v>10</v>
+      </c>
+      <c r="G433">
+        <v>1</v>
+      </c>
+      <c r="H433">
+        <v>90</v>
+      </c>
+      <c r="I433">
+        <v>1</v>
+      </c>
+      <c r="J433">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="434" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A434">
+        <v>22</v>
+      </c>
+      <c r="B434" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C434">
+        <v>22</v>
+      </c>
+      <c r="D434" t="s">
+        <v>51</v>
+      </c>
+      <c r="F434">
+        <v>10</v>
+      </c>
+      <c r="G434">
+        <v>1</v>
+      </c>
+      <c r="H434">
+        <v>90</v>
+      </c>
+      <c r="I434">
+        <v>1</v>
+      </c>
+      <c r="J434">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -12413,13 +12868,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFDCF622-BAB6-4971-B843-0A581D15DC9C}">
   <dimension ref="A1:R23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -12475,7 +12930,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -12534,7 +12989,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -12575,15 +13030,15 @@
         <v>0</v>
       </c>
       <c r="N3">
-        <f t="shared" ref="N3:N22" si="0">SUM(H3:I3)</f>
+        <f t="shared" ref="N3:N23" si="0">SUM(H3:I3)</f>
         <v>1</v>
       </c>
       <c r="O3">
-        <f t="shared" ref="O3:O22" si="1">SUM(J3:K3)</f>
+        <f t="shared" ref="O3:O23" si="1">SUM(J3:K3)</f>
         <v>0</v>
       </c>
       <c r="P3">
-        <f t="shared" ref="P3:P22" si="2">SUM(L3:M3)</f>
+        <f t="shared" ref="P3:P23" si="2">SUM(L3:M3)</f>
         <v>1</v>
       </c>
       <c r="Q3">
@@ -12593,7 +13048,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -12652,7 +13107,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -12711,7 +13166,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -12770,7 +13225,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -12829,7 +13284,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -12888,7 +13343,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -12947,7 +13402,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -13006,7 +13461,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -13065,7 +13520,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -13124,7 +13579,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -13183,7 +13638,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -13242,7 +13697,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -13301,7 +13756,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -13360,7 +13815,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -13419,7 +13874,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -13478,7 +13933,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -13537,7 +13992,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -13596,7 +14051,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -13655,7 +14110,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -13714,8 +14169,64 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="B23" s="1"/>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" s="1">
+        <v>46103</v>
+      </c>
+      <c r="C23" s="5">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="D23">
+        <v>10</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>1</v>
+      </c>
+      <c r="G23">
+        <v>1</v>
+      </c>
+      <c r="H23">
+        <v>5</v>
+      </c>
+      <c r="I23">
+        <v>4</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>1</v>
+      </c>
+      <c r="L23">
+        <v>5</v>
+      </c>
+      <c r="M23">
+        <v>7</v>
+      </c>
+      <c r="N23">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="O23">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="P23">
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="Q23">
+        <v>28</v>
+      </c>
+      <c r="R23">
+        <v>11</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13725,12 +14236,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B5D582A-AEC7-431B-9531-7497C8635E57}">
   <dimension ref="A1:B17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="35.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -13738,7 +14249,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -13746,7 +14257,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>11</v>
       </c>
@@ -13754,7 +14265,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -13762,7 +14273,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -13770,7 +14281,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -13778,7 +14289,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -13786,7 +14297,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -13794,7 +14305,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -13802,7 +14313,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -13810,7 +14321,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -13818,7 +14329,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2</v>
       </c>
@@ -13826,7 +14337,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -13834,7 +14345,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -13842,7 +14353,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -13850,7 +14361,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -13858,7 +14369,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>

</xml_diff>